<commit_message>
Remove chart objects (Donut/Bar) to fix Excel content-repair error; keep COUNTIF summary + KPIs; prefix FILTER with _xlfn._xlws
</commit_message>
<xml_diff>
--- a/SAP_PM_ECC6_to_S4_Migration.xlsx
+++ b/SAP_PM_ECC6_to_S4_Migration.xlsx
@@ -973,255 +973,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>התקדמות לפי סטטוס</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Cockpit מעקב מיגרציה'!L2</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Cockpit מעקב מיגרציה'!$K$3:$K$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit מעקב מיגרציה'!$L$3:$L$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>התפלגות סטטוס מיגרציה</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <doughnutChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Cockpit מעקב מיגרציה'!L2</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <dPt>
-            <idx val="0"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="FCE4E6"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="1"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="ECEFF1"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="2"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="E1E6EA"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="3"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="DCE6EC"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="4"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="DCEFE0"/>
-              </a:solidFill>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <cat>
-            <numRef>
-              <f>'Cockpit מעקב מיגרציה'!$K$3:$K$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit מעקב מיגרציה'!$L$3:$L$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showVal val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-        <holeSize val="55"/>
-      </doughnutChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>9</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3960000" cy="1872000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>10</col>
-      <colOff>0</colOff>
-      <row>10</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3960000" cy="2700000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3079,7 +2830,7 @@
     <row r="28">
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="33">
-        <f>IF(C25="","הקלד מונח בתא הצהוב למעלה - והתוצאות יופיעו כאן מיד (כולל קישור לחיץ)...",IFERROR(FILTER(CHOOSE({1,2,3,4,5,6},$V$2:$V$768,$Q$2:$Q$768,$R$2:$R$768,$S$2:$S$768,$T$2:$T$768,$U$2:$U$768),(ISNUMBER(SEARCH(C25,$Q$2:$Q$768)))+(ISNUMBER(SEARCH(C25,$R$2:$R$768)))+(ISNUMBER(SEARCH(C25,$S$2:$S$768)))+(ISNUMBER(SEARCH(C25,$P$2:$P$768)))&gt;0),"לא נמצאו תוצאות - נסה מונח אחר"))</f>
+        <f>IF(C25="","הקלד מונח בתא הצהוב למעלה - והתוצאות יופיעו כאן מיד (כולל קישור לחיץ)...",IFERROR(_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6},$V$2:$V$768,$Q$2:$Q$768,$R$2:$R$768,$S$2:$S$768,$T$2:$T$768,$U$2:$U$768),(ISNUMBER(SEARCH(C25,$Q$2:$Q$768)))+(ISNUMBER(SEARCH(C25,$R$2:$R$768)))+(ISNUMBER(SEARCH(C25,$S$2:$S$768)))+(ISNUMBER(SEARCH(C25,$P$2:$P$768)))&gt;0),"לא נמצאו תוצאות - נסה מונח אחר"))</f>
         <v/>
       </c>
       <c r="C28" s="1" t="n"/>
@@ -40745,7 +40496,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
 </worksheet>
 </file>
 
@@ -49106,7 +48856,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add JOIN ON (SQL syntax) column to ER Map in monospace Consolas; preserve Consolas through font post-pass
</commit_message>
<xml_diff>
--- a/SAP_PM_ECC6_to_S4_Migration.xlsx
+++ b/SAP_PM_ECC6_to_S4_Migration.xlsx
@@ -58,7 +58,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="15">'Custom Code Check'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="15">'Custom Code Check'!$A$1:$I$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="16">'ER - Join Map'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="16">'ER - Join Map'!$A$1:$I$60</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="16">'ER - Join Map'!$A$1:$J$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +67,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="63">
+  <fonts count="64">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -262,6 +262,12 @@
       <color rgb="000563C1"/>
       <sz val="9"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000B5394"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -605,51 +611,51 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="54" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="55" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="55" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="39" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="40" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -676,33 +682,33 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="43" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="60" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="12" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="61" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="61" fillId="12" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="62" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="63" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="54" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -745,7 +751,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -764,7 +770,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -900,8 +906,14 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -44631,7 +44643,7 @@
       </c>
       <c r="Q849" s="8" t="inlineStr">
         <is>
-          <t>IFLOS.TPLNR -&gt; IFLOT.TPLNR</t>
+          <t>IFLOS.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R849" s="7" t="inlineStr">
@@ -44678,7 +44690,7 @@
       </c>
       <c r="Q850" s="8" t="inlineStr">
         <is>
-          <t>IFLOT.TPLMA -&gt; IFLOT.TPLNR</t>
+          <t>IFLOT.TPLMA = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R850" s="7" t="inlineStr">
@@ -44725,7 +44737,7 @@
       </c>
       <c r="Q851" s="8" t="inlineStr">
         <is>
-          <t>IFLOT.OBJNR -&gt; JSTO.OBJNR</t>
+          <t>IFLOT.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R851" s="7" t="inlineStr">
@@ -44772,7 +44784,7 @@
       </c>
       <c r="Q852" s="8" t="inlineStr">
         <is>
-          <t>ILOA.TPLNR -&gt; IFLOT.TPLNR</t>
+          <t>ILOA.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R852" s="7" t="inlineStr">
@@ -44819,7 +44831,7 @@
       </c>
       <c r="Q853" s="8" t="inlineStr">
         <is>
-          <t>ILOA.GEWRK -&gt; CRHD.OBJID</t>
+          <t>ILOA.GEWRK = CRHD.OBJID</t>
         </is>
       </c>
       <c r="R853" s="7" t="inlineStr">
@@ -44866,7 +44878,7 @@
       </c>
       <c r="Q854" s="8" t="inlineStr">
         <is>
-          <t>CRTX.OBJID -&gt; CRHD.OBJID</t>
+          <t>CRTX.OBJID = CRHD.OBJID</t>
         </is>
       </c>
       <c r="R854" s="7" t="inlineStr">
@@ -44913,7 +44925,7 @@
       </c>
       <c r="Q855" s="8" t="inlineStr">
         <is>
-          <t>EQKT.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>EQKT.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R855" s="7" t="inlineStr">
@@ -44960,7 +44972,7 @@
       </c>
       <c r="Q856" s="8" t="inlineStr">
         <is>
-          <t>EQUZ.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>EQUZ.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R856" s="7" t="inlineStr">
@@ -45007,7 +45019,7 @@
       </c>
       <c r="Q857" s="8" t="inlineStr">
         <is>
-          <t>EQUZ.HEQUI -&gt; EQUI.EQUNR</t>
+          <t>EQUZ.HEQUI = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R857" s="7" t="inlineStr">
@@ -45054,7 +45066,7 @@
       </c>
       <c r="Q858" s="8" t="inlineStr">
         <is>
-          <t>EQUZ.ILOAN -&gt; ILOA.ILOAN</t>
+          <t>EQUZ.ILOAN = ILOA.ILOAN</t>
         </is>
       </c>
       <c r="R858" s="7" t="inlineStr">
@@ -45101,7 +45113,7 @@
       </c>
       <c r="Q859" s="8" t="inlineStr">
         <is>
-          <t>EQUI.OBJNR -&gt; JSTO.OBJNR</t>
+          <t>EQUI.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R859" s="7" t="inlineStr">
@@ -45148,7 +45160,7 @@
       </c>
       <c r="Q860" s="8" t="inlineStr">
         <is>
-          <t>OBJK.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>OBJK.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R860" s="7" t="inlineStr">
@@ -45195,7 +45207,7 @@
       </c>
       <c r="Q861" s="8" t="inlineStr">
         <is>
-          <t>STPO.STLNR -&gt; STKO.STLNR</t>
+          <t>STPO.STLNR = STKO.STLNR</t>
         </is>
       </c>
       <c r="R861" s="7" t="inlineStr">
@@ -45242,7 +45254,7 @@
       </c>
       <c r="Q862" s="8" t="inlineStr">
         <is>
-          <t>MAST.STLNR -&gt; STKO.STLNR</t>
+          <t>MAST.STLNR = STKO.STLNR</t>
         </is>
       </c>
       <c r="R862" s="7" t="inlineStr">
@@ -45289,7 +45301,7 @@
       </c>
       <c r="Q863" s="8" t="inlineStr">
         <is>
-          <t>EQST.STLNR -&gt; STKO.STLNR</t>
+          <t>EQST.STLNR = STKO.STLNR</t>
         </is>
       </c>
       <c r="R863" s="7" t="inlineStr">
@@ -45336,7 +45348,7 @@
       </c>
       <c r="Q864" s="8" t="inlineStr">
         <is>
-          <t>EQST.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>EQST.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R864" s="7" t="inlineStr">
@@ -45383,7 +45395,7 @@
       </c>
       <c r="Q865" s="8" t="inlineStr">
         <is>
-          <t>TPST.STLNR -&gt; STKO.STLNR</t>
+          <t>TPST.STLNR = STKO.STLNR</t>
         </is>
       </c>
       <c r="R865" s="7" t="inlineStr">
@@ -45430,7 +45442,7 @@
       </c>
       <c r="Q866" s="8" t="inlineStr">
         <is>
-          <t>TPST.TPLNR -&gt; IFLOT.TPLNR</t>
+          <t>TPST.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R866" s="7" t="inlineStr">
@@ -45477,7 +45489,7 @@
       </c>
       <c r="Q867" s="8" t="inlineStr">
         <is>
-          <t>IMRG.POINT -&gt; IMPTT.POINT</t>
+          <t>IMRG.POINT = IMPTT.POINT</t>
         </is>
       </c>
       <c r="R867" s="7" t="inlineStr">
@@ -45524,7 +45536,7 @@
       </c>
       <c r="Q868" s="8" t="inlineStr">
         <is>
-          <t>QPCD.CODEGRUPPE -&gt; QPGR.CODEGRUPPE</t>
+          <t>QPCD.CODEGRUPPE = QPGR.CODEGRUPPE</t>
         </is>
       </c>
       <c r="R868" s="7" t="inlineStr">
@@ -45571,7 +45583,7 @@
       </c>
       <c r="Q869" s="8" t="inlineStr">
         <is>
-          <t>T352B.CODEGRUPPE -&gt; QPGR.CODEGRUPPE</t>
+          <t>T352B.CODEGRUPPE = QPGR.CODEGRUPPE</t>
         </is>
       </c>
       <c r="R869" s="7" t="inlineStr">
@@ -45618,7 +45630,7 @@
       </c>
       <c r="Q870" s="8" t="inlineStr">
         <is>
-          <t>QMFE.QMNUM -&gt; QMEL.QMNUM</t>
+          <t>QMFE.QMNUM = QMEL.QMNUM</t>
         </is>
       </c>
       <c r="R870" s="7" t="inlineStr">
@@ -45665,7 +45677,7 @@
       </c>
       <c r="Q871" s="8" t="inlineStr">
         <is>
-          <t>QMUR.QMNUM -&gt; QMFE.QMNUM</t>
+          <t>QMUR.QMNUM = QMFE.QMNUM</t>
         </is>
       </c>
       <c r="R871" s="7" t="inlineStr">
@@ -45712,7 +45724,7 @@
       </c>
       <c r="Q872" s="8" t="inlineStr">
         <is>
-          <t>QMMA.QMNUM -&gt; QMEL.QMNUM</t>
+          <t>QMMA.QMNUM = QMEL.QMNUM</t>
         </is>
       </c>
       <c r="R872" s="7" t="inlineStr">
@@ -45759,7 +45771,7 @@
       </c>
       <c r="Q873" s="8" t="inlineStr">
         <is>
-          <t>QMSM.QMNUM -&gt; QMEL.QMNUM</t>
+          <t>QMSM.QMNUM = QMEL.QMNUM</t>
         </is>
       </c>
       <c r="R873" s="7" t="inlineStr">
@@ -45806,7 +45818,7 @@
       </c>
       <c r="Q874" s="8" t="inlineStr">
         <is>
-          <t>QMEL.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>QMEL.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R874" s="7" t="inlineStr">
@@ -45853,7 +45865,7 @@
       </c>
       <c r="Q875" s="8" t="inlineStr">
         <is>
-          <t>QMEL.TPLNR -&gt; IFLOT.TPLNR</t>
+          <t>QMEL.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R875" s="7" t="inlineStr">
@@ -45900,7 +45912,7 @@
       </c>
       <c r="Q876" s="8" t="inlineStr">
         <is>
-          <t>QMEL.OBJNR -&gt; JSTO.OBJNR</t>
+          <t>QMEL.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R876" s="7" t="inlineStr">
@@ -45947,7 +45959,7 @@
       </c>
       <c r="Q877" s="8" t="inlineStr">
         <is>
-          <t>QMEL.QMART -&gt; TQ80.QMART</t>
+          <t>QMEL.QMART = TQ80.QMART</t>
         </is>
       </c>
       <c r="R877" s="7" t="inlineStr">
@@ -45994,7 +46006,7 @@
       </c>
       <c r="Q878" s="8" t="inlineStr">
         <is>
-          <t>AFKO.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>AFKO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R878" s="7" t="inlineStr">
@@ -46041,7 +46053,7 @@
       </c>
       <c r="Q879" s="8" t="inlineStr">
         <is>
-          <t>AFPO.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>AFPO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R879" s="7" t="inlineStr">
@@ -46088,7 +46100,7 @@
       </c>
       <c r="Q880" s="8" t="inlineStr">
         <is>
-          <t>AFIH.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>AFIH.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R880" s="7" t="inlineStr">
@@ -46135,7 +46147,7 @@
       </c>
       <c r="Q881" s="8" t="inlineStr">
         <is>
-          <t>AFVC.AUFPL -&gt; AFKO.AUFPL</t>
+          <t>AFVC.AUFPL = AFKO.AUFPL</t>
         </is>
       </c>
       <c r="R881" s="7" t="inlineStr">
@@ -46182,7 +46194,7 @@
       </c>
       <c r="Q882" s="8" t="inlineStr">
         <is>
-          <t>AFVC.ARBID -&gt; CRHD.OBJID</t>
+          <t>AFVC.ARBID = CRHD.OBJID</t>
         </is>
       </c>
       <c r="R882" s="7" t="inlineStr">
@@ -46229,7 +46241,7 @@
       </c>
       <c r="Q883" s="8" t="inlineStr">
         <is>
-          <t>AFIH.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>AFIH.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R883" s="7" t="inlineStr">
@@ -46276,7 +46288,7 @@
       </c>
       <c r="Q884" s="8" t="inlineStr">
         <is>
-          <t>AFIH.TPLNR -&gt; IFLOT.TPLNR</t>
+          <t>AFIH.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R884" s="7" t="inlineStr">
@@ -46323,7 +46335,7 @@
       </c>
       <c r="Q885" s="8" t="inlineStr">
         <is>
-          <t>AUFK.OBJNR -&gt; JSTO.OBJNR</t>
+          <t>AUFK.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R885" s="7" t="inlineStr">
@@ -46370,7 +46382,7 @@
       </c>
       <c r="Q886" s="8" t="inlineStr">
         <is>
-          <t>AUFK.AUART -&gt; T003O.AUART</t>
+          <t>AUFK.AUART = T003O.AUART</t>
         </is>
       </c>
       <c r="R886" s="7" t="inlineStr">
@@ -46417,7 +46429,7 @@
       </c>
       <c r="Q887" s="8" t="inlineStr">
         <is>
-          <t>JEST.OBJNR -&gt; JSTO.OBJNR</t>
+          <t>JEST.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R887" s="7" t="inlineStr">
@@ -46464,7 +46476,7 @@
       </c>
       <c r="Q888" s="8" t="inlineStr">
         <is>
-          <t>JSTO.STSMA -&gt; TJ30.STSMA</t>
+          <t>JSTO.STSMA = TJ30.STSMA</t>
         </is>
       </c>
       <c r="R888" s="7" t="inlineStr">
@@ -46511,7 +46523,7 @@
       </c>
       <c r="Q889" s="8" t="inlineStr">
         <is>
-          <t>T003O.STSMA -&gt; TJ30.STSMA</t>
+          <t>T003O.STSMA = TJ30.STSMA</t>
         </is>
       </c>
       <c r="R889" s="7" t="inlineStr">
@@ -46558,7 +46570,7 @@
       </c>
       <c r="Q890" s="8" t="inlineStr">
         <is>
-          <t>RESB.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>RESB.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R890" s="7" t="inlineStr">
@@ -46605,7 +46617,7 @@
       </c>
       <c r="Q891" s="8" t="inlineStr">
         <is>
-          <t>MSEG.MBLNR -&gt; MKPF.MBLNR</t>
+          <t>MSEG.MBLNR = MKPF.MBLNR</t>
         </is>
       </c>
       <c r="R891" s="7" t="inlineStr">
@@ -46652,7 +46664,7 @@
       </c>
       <c r="Q892" s="8" t="inlineStr">
         <is>
-          <t>MSEG.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>MSEG.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R892" s="7" t="inlineStr">
@@ -46699,7 +46711,7 @@
       </c>
       <c r="Q893" s="8" t="inlineStr">
         <is>
-          <t>EBKN.BANFN -&gt; EBAN.BANFN</t>
+          <t>EBKN.BANFN = EBAN.BANFN</t>
         </is>
       </c>
       <c r="R893" s="7" t="inlineStr">
@@ -46746,7 +46758,7 @@
       </c>
       <c r="Q894" s="8" t="inlineStr">
         <is>
-          <t>EBKN.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>EBKN.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R894" s="7" t="inlineStr">
@@ -46793,7 +46805,7 @@
       </c>
       <c r="Q895" s="8" t="inlineStr">
         <is>
-          <t>COSP.OBJNR -&gt; AUFK.OBJNR</t>
+          <t>COSP.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="R895" s="7" t="inlineStr">
@@ -46840,7 +46852,7 @@
       </c>
       <c r="Q896" s="8" t="inlineStr">
         <is>
-          <t>COSS.OBJNR -&gt; AUFK.OBJNR</t>
+          <t>COSS.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="R896" s="7" t="inlineStr">
@@ -46887,7 +46899,7 @@
       </c>
       <c r="Q897" s="8" t="inlineStr">
         <is>
-          <t>COBRA.OBJNR -&gt; AUFK.OBJNR</t>
+          <t>COBRA.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="R897" s="7" t="inlineStr">
@@ -46934,7 +46946,7 @@
       </c>
       <c r="Q898" s="8" t="inlineStr">
         <is>
-          <t>COBRB.OBJNR -&gt; COBRA.OBJNR</t>
+          <t>COBRB.OBJNR = COBRA.OBJNR</t>
         </is>
       </c>
       <c r="R898" s="7" t="inlineStr">
@@ -46981,7 +46993,7 @@
       </c>
       <c r="Q899" s="8" t="inlineStr">
         <is>
-          <t>MPOS.WARPL -&gt; MPLA.WARPL</t>
+          <t>MPOS.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="R899" s="7" t="inlineStr">
@@ -47028,7 +47040,7 @@
       </c>
       <c r="Q900" s="8" t="inlineStr">
         <is>
-          <t>MPOS.EQUNR -&gt; EQUI.EQUNR</t>
+          <t>MPOS.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R900" s="7" t="inlineStr">
@@ -47075,7 +47087,7 @@
       </c>
       <c r="Q901" s="8" t="inlineStr">
         <is>
-          <t>MPOS.PLNNR -&gt; PLKO.PLNNR</t>
+          <t>MPOS.PLNNR = PLKO.PLNNR</t>
         </is>
       </c>
       <c r="R901" s="7" t="inlineStr">
@@ -47122,7 +47134,7 @@
       </c>
       <c r="Q902" s="8" t="inlineStr">
         <is>
-          <t>MHIO.WARPL -&gt; MPLA.WARPL</t>
+          <t>MHIO.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="R902" s="7" t="inlineStr">
@@ -47169,7 +47181,7 @@
       </c>
       <c r="Q903" s="8" t="inlineStr">
         <is>
-          <t>MHIO.AUFNR -&gt; AUFK.AUFNR</t>
+          <t>MHIO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R903" s="7" t="inlineStr">
@@ -47216,7 +47228,7 @@
       </c>
       <c r="Q904" s="8" t="inlineStr">
         <is>
-          <t>MHIS.WARPL -&gt; MPLA.WARPL</t>
+          <t>MHIS.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="R904" s="7" t="inlineStr">
@@ -47263,7 +47275,7 @@
       </c>
       <c r="Q905" s="8" t="inlineStr">
         <is>
-          <t>PLPO.PLNNR -&gt; PLKO.PLNNR</t>
+          <t>PLPO.PLNNR = PLKO.PLNNR</t>
         </is>
       </c>
       <c r="R905" s="7" t="inlineStr">
@@ -47310,7 +47322,7 @@
       </c>
       <c r="Q906" s="8" t="inlineStr">
         <is>
-          <t>PLPO.ARBID -&gt; CRHD.OBJID</t>
+          <t>PLPO.ARBID = CRHD.OBJID</t>
         </is>
       </c>
       <c r="R906" s="7" t="inlineStr">
@@ -58733,7 +58745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -58743,8 +58755,9 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -58765,6 +58778,7 @@
       <c r="G1" s="4" t="n"/>
       <c r="H1" s="4" t="n"/>
       <c r="I1" s="4" t="n"/>
+      <c r="J1" s="4" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="73" t="inlineStr">
@@ -58804,10 +58818,15 @@
       </c>
       <c r="H2" s="73" t="inlineStr">
         <is>
+          <t>JOIN ON (SQL syntax)</t>
+        </is>
+      </c>
+      <c r="I2" s="73" t="inlineStr">
+        <is>
           <t>תיאור הקשר (Hebrew)</t>
         </is>
       </c>
-      <c r="I2" s="73" t="inlineStr">
+      <c r="J2" s="73" t="inlineStr">
         <is>
           <t>מעבר לטבלה</t>
         </is>
@@ -58847,12 +58866,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H3" s="46" t="inlineStr">
+      <c r="H3" s="104" t="inlineStr">
+        <is>
+          <t>IFLOS.TPLNR = IFLOT.TPLNR</t>
+        </is>
+      </c>
+      <c r="I3" s="46" t="inlineStr">
         <is>
           <t>תווית מיקום פונקציונלי מצורפת לרשומת האב</t>
         </is>
       </c>
-      <c r="I3" s="104">
+      <c r="J3" s="105">
         <f>HYPERLINK("#'"&amp;"1. מבנה ארגוני ותשתית"&amp;"'!A11","➜ פתח")</f>
         <v/>
       </c>
@@ -58891,12 +58915,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H4" s="54" t="inlineStr">
+      <c r="H4" s="106" t="inlineStr">
+        <is>
+          <t>IFLOT.TPLMA = IFLOT.TPLNR</t>
+        </is>
+      </c>
+      <c r="I4" s="54" t="inlineStr">
         <is>
           <t>היררכיית מיקומים - מיקום אב (self-join)</t>
         </is>
       </c>
-      <c r="I4" s="105">
+      <c r="J4" s="107">
         <f>HYPERLINK("#'"&amp;"1. מבנה ארגוני ותשתית"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -58935,12 +58964,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H5" s="46" t="inlineStr">
+      <c r="H5" s="104" t="inlineStr">
+        <is>
+          <t>IFLOT.OBJNR = JSTO.OBJNR</t>
+        </is>
+      </c>
+      <c r="I5" s="46" t="inlineStr">
         <is>
           <t>אובייקט הסטטוס של המיקום הפונקציונלי</t>
         </is>
       </c>
-      <c r="I5" s="104">
+      <c r="J5" s="105">
         <f>HYPERLINK("#'"&amp;"1. מבנה ארגוני ותשתית"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -58979,12 +59013,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H6" s="54" t="inlineStr">
+      <c r="H6" s="106" t="inlineStr">
+        <is>
+          <t>ILOA.TPLNR = IFLOT.TPLNR</t>
+        </is>
+      </c>
+      <c r="I6" s="54" t="inlineStr">
         <is>
           <t>נתוני מיקום/חיוב משויכים למיקום הפונקציונלי</t>
         </is>
       </c>
-      <c r="I6" s="105">
+      <c r="J6" s="107">
         <f>HYPERLINK("#'"&amp;"1. מבנה ארגוני ותשתית"&amp;"'!A18","➜ פתח")</f>
         <v/>
       </c>
@@ -59023,12 +59062,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H7" s="46" t="inlineStr">
+      <c r="H7" s="104" t="inlineStr">
+        <is>
+          <t>ILOA.GEWRK = CRHD.OBJID</t>
+        </is>
+      </c>
+      <c r="I7" s="46" t="inlineStr">
         <is>
           <t>מרכז עבודה ראשי אחראי</t>
         </is>
       </c>
-      <c r="I7" s="104">
+      <c r="J7" s="105">
         <f>HYPERLINK("#'"&amp;"1. מבנה ארגוני ותשתית"&amp;"'!A18","➜ פתח")</f>
         <v/>
       </c>
@@ -59067,12 +59111,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H8" s="54" t="inlineStr">
+      <c r="H8" s="106" t="inlineStr">
+        <is>
+          <t>CRTX.OBJID = CRHD.OBJID</t>
+        </is>
+      </c>
+      <c r="I8" s="54" t="inlineStr">
         <is>
           <t>טקסטים של מרכז העבודה (לפי שפה)</t>
         </is>
       </c>
-      <c r="I8" s="105">
+      <c r="J8" s="107">
         <f>HYPERLINK("#'"&amp;"1. מבנה ארגוני ותשתית"&amp;"'!A34","➜ פתח")</f>
         <v/>
       </c>
@@ -59111,12 +59160,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H9" s="46" t="inlineStr">
+      <c r="H9" s="104" t="inlineStr">
+        <is>
+          <t>EQKT.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I9" s="46" t="inlineStr">
         <is>
           <t>טקסטים של הציוד (לפי שפה)</t>
         </is>
       </c>
-      <c r="I9" s="104">
+      <c r="J9" s="105">
         <f>HYPERLINK("#'"&amp;"2. ציוד ונתוני מאסטר"&amp;"'!A11","➜ פתח")</f>
         <v/>
       </c>
@@ -59155,12 +59209,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H10" s="54" t="inlineStr">
+      <c r="H10" s="106" t="inlineStr">
+        <is>
+          <t>EQUZ.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I10" s="54" t="inlineStr">
         <is>
           <t>פלחי זמן של הציוד (התקנות לאורך זמן)</t>
         </is>
       </c>
-      <c r="I10" s="105">
+      <c r="J10" s="107">
         <f>HYPERLINK("#'"&amp;"2. ציוד ונתוני מאסטר"&amp;"'!A16","➜ פתח")</f>
         <v/>
       </c>
@@ -59199,12 +59258,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H11" s="46" t="inlineStr">
+      <c r="H11" s="104" t="inlineStr">
+        <is>
+          <t>EQUZ.HEQUI = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr">
         <is>
           <t>ציוד עליון בהיררכיה (self-join דרך EQUI)</t>
         </is>
       </c>
-      <c r="I11" s="104">
+      <c r="J11" s="105">
         <f>HYPERLINK("#'"&amp;"2. ציוד ונתוני מאסטר"&amp;"'!A16","➜ פתח")</f>
         <v/>
       </c>
@@ -59243,12 +59307,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H12" s="54" t="inlineStr">
+      <c r="H12" s="106" t="inlineStr">
+        <is>
+          <t>EQUZ.ILOAN = ILOA.ILOAN</t>
+        </is>
+      </c>
+      <c r="I12" s="54" t="inlineStr">
         <is>
           <t>נתוני מיקום/חיוב של הציוד בפלח הזמן</t>
         </is>
       </c>
-      <c r="I12" s="105">
+      <c r="J12" s="107">
         <f>HYPERLINK("#'"&amp;"2. ציוד ונתוני מאסטר"&amp;"'!A16","➜ פתח")</f>
         <v/>
       </c>
@@ -59287,12 +59356,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H13" s="46" t="inlineStr">
+      <c r="H13" s="104" t="inlineStr">
+        <is>
+          <t>EQUI.OBJNR = JSTO.OBJNR</t>
+        </is>
+      </c>
+      <c r="I13" s="46" t="inlineStr">
         <is>
           <t>אובייקט הסטטוס של הציוד</t>
         </is>
       </c>
-      <c r="I13" s="104">
+      <c r="J13" s="105">
         <f>HYPERLINK("#'"&amp;"2. ציוד ונתוני מאסטר"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -59331,12 +59405,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H14" s="54" t="inlineStr">
+      <c r="H14" s="106" t="inlineStr">
+        <is>
+          <t>OBJK.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I14" s="54" t="inlineStr">
         <is>
           <t>מספר סידורי משויך לרשומת ציוד</t>
         </is>
       </c>
-      <c r="I14" s="105">
+      <c r="J14" s="107">
         <f>HYPERLINK("#'"&amp;"2. ציוד ונתוני מאסטר"&amp;"'!A23","➜ פתח")</f>
         <v/>
       </c>
@@ -59375,12 +59454,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
+      <c r="H15" s="104" t="inlineStr">
+        <is>
+          <t>STPO.STLNR = STKO.STLNR</t>
+        </is>
+      </c>
+      <c r="I15" s="46" t="inlineStr">
         <is>
           <t>פריטי עץ המוצר תחת הכותרת</t>
         </is>
       </c>
-      <c r="I15" s="104">
+      <c r="J15" s="105">
         <f>HYPERLINK("#'"&amp;"3. עצי מוצר של אחזקה (BOM)"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
@@ -59419,12 +59503,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H16" s="54" t="inlineStr">
+      <c r="H16" s="106" t="inlineStr">
+        <is>
+          <t>MAST.STLNR = STKO.STLNR</t>
+        </is>
+      </c>
+      <c r="I16" s="54" t="inlineStr">
         <is>
           <t>קישור חומר לכותרת עץ המוצר</t>
         </is>
       </c>
-      <c r="I16" s="105">
+      <c r="J16" s="107">
         <f>HYPERLINK("#'"&amp;"3. עצי מוצר של אחזקה (BOM)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
@@ -59463,12 +59552,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H17" s="46" t="inlineStr">
+      <c r="H17" s="104" t="inlineStr">
+        <is>
+          <t>EQST.STLNR = STKO.STLNR</t>
+        </is>
+      </c>
+      <c r="I17" s="46" t="inlineStr">
         <is>
           <t>קישור ציוד לעץ המוצר</t>
         </is>
       </c>
-      <c r="I17" s="104">
+      <c r="J17" s="105">
         <f>HYPERLINK("#'"&amp;"3. עצי מוצר של אחזקה (BOM)"&amp;"'!A24","➜ פתח")</f>
         <v/>
       </c>
@@ -59507,12 +59601,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H18" s="54" t="inlineStr">
+      <c r="H18" s="106" t="inlineStr">
+        <is>
+          <t>EQST.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I18" s="54" t="inlineStr">
         <is>
           <t>עץ המוצר של הציוד</t>
         </is>
       </c>
-      <c r="I18" s="105">
+      <c r="J18" s="107">
         <f>HYPERLINK("#'"&amp;"3. עצי מוצר של אחזקה (BOM)"&amp;"'!A24","➜ פתח")</f>
         <v/>
       </c>
@@ -59551,12 +59650,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H19" s="46" t="inlineStr">
+      <c r="H19" s="104" t="inlineStr">
+        <is>
+          <t>TPST.STLNR = STKO.STLNR</t>
+        </is>
+      </c>
+      <c r="I19" s="46" t="inlineStr">
         <is>
           <t>קישור מיקום לעץ המוצר</t>
         </is>
       </c>
-      <c r="I19" s="104">
+      <c r="J19" s="105">
         <f>HYPERLINK("#'"&amp;"3. עצי מוצר של אחזקה (BOM)"&amp;"'!A30","➜ פתח")</f>
         <v/>
       </c>
@@ -59595,12 +59699,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H20" s="54" t="inlineStr">
+      <c r="H20" s="106" t="inlineStr">
+        <is>
+          <t>TPST.TPLNR = IFLOT.TPLNR</t>
+        </is>
+      </c>
+      <c r="I20" s="54" t="inlineStr">
         <is>
           <t>עץ המוצר של המיקום הפונקציונלי</t>
         </is>
       </c>
-      <c r="I20" s="105">
+      <c r="J20" s="107">
         <f>HYPERLINK("#'"&amp;"3. עצי מוצר של אחזקה (BOM)"&amp;"'!A30","➜ פתח")</f>
         <v/>
       </c>
@@ -59639,12 +59748,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H21" s="46" t="inlineStr">
+      <c r="H21" s="104" t="inlineStr">
+        <is>
+          <t>IMRG.POINT = IMPTT.POINT</t>
+        </is>
+      </c>
+      <c r="I21" s="46" t="inlineStr">
         <is>
           <t>מסמכי מדידה תחת נקודת המדידה</t>
         </is>
       </c>
-      <c r="I21" s="104">
+      <c r="J21" s="105">
         <f>HYPERLINK("#'"&amp;"4. נקודות מדידה ומונים"&amp;"'!A11","➜ פתח")</f>
         <v/>
       </c>
@@ -59683,12 +59797,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H22" s="54" t="inlineStr">
+      <c r="H22" s="106" t="inlineStr">
+        <is>
+          <t>QPCD.CODEGRUPPE = QPGR.CODEGRUPPE</t>
+        </is>
+      </c>
+      <c r="I22" s="54" t="inlineStr">
         <is>
           <t>קודים בתוך קבוצת הקוד</t>
         </is>
       </c>
-      <c r="I22" s="105">
+      <c r="J22" s="107">
         <f>HYPERLINK("#'"&amp;"5. קטלוגים, קודים ופרופילים"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -59727,12 +59846,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H23" s="46" t="inlineStr">
+      <c r="H23" s="104" t="inlineStr">
+        <is>
+          <t>T352B.CODEGRUPPE = QPGR.CODEGRUPPE</t>
+        </is>
+      </c>
+      <c r="I23" s="46" t="inlineStr">
         <is>
           <t>קבוצות קוד מותרות בפרופיל הקטלוג</t>
         </is>
       </c>
-      <c r="I23" s="104">
+      <c r="J23" s="105">
         <f>HYPERLINK("#'"&amp;"5. קטלוגים, קודים ופרופילים"&amp;"'!A15","➜ פתח")</f>
         <v/>
       </c>
@@ -59771,12 +59895,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H24" s="54" t="inlineStr">
+      <c r="H24" s="106" t="inlineStr">
+        <is>
+          <t>QMFE.QMNUM = QMEL.QMNUM</t>
+        </is>
+      </c>
+      <c r="I24" s="54" t="inlineStr">
         <is>
           <t>פריטי הליקוי תחת ההודעה</t>
         </is>
       </c>
-      <c r="I24" s="105">
+      <c r="J24" s="107">
         <f>HYPERLINK("#'"&amp;"6. הודעות אחזקה (Notifications)"&amp;"'!A11","➜ פתח")</f>
         <v/>
       </c>
@@ -59815,12 +59944,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H25" s="46" t="inlineStr">
+      <c r="H25" s="104" t="inlineStr">
+        <is>
+          <t>QMUR.QMNUM = QMFE.QMNUM</t>
+        </is>
+      </c>
+      <c r="I25" s="46" t="inlineStr">
         <is>
           <t>סיבות תחת פריט ההודעה (דרך QMNUM+FENUM)</t>
         </is>
       </c>
-      <c r="I25" s="104">
+      <c r="J25" s="105">
         <f>HYPERLINK("#'"&amp;"6. הודעות אחזקה (Notifications)"&amp;"'!A19","➜ פתח")</f>
         <v/>
       </c>
@@ -59859,12 +59993,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H26" s="54" t="inlineStr">
+      <c r="H26" s="106" t="inlineStr">
+        <is>
+          <t>QMMA.QMNUM = QMEL.QMNUM</t>
+        </is>
+      </c>
+      <c r="I26" s="54" t="inlineStr">
         <is>
           <t>פעילויות שבוצעו תחת ההודעה</t>
         </is>
       </c>
-      <c r="I26" s="105">
+      <c r="J26" s="107">
         <f>HYPERLINK("#'"&amp;"6. הודעות אחזקה (Notifications)"&amp;"'!A26","➜ פתח")</f>
         <v/>
       </c>
@@ -59903,12 +60042,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H27" s="46" t="inlineStr">
+      <c r="H27" s="104" t="inlineStr">
+        <is>
+          <t>QMSM.QMNUM = QMEL.QMNUM</t>
+        </is>
+      </c>
+      <c r="I27" s="46" t="inlineStr">
         <is>
           <t>משימות לטיפול תחת ההודעה</t>
         </is>
       </c>
-      <c r="I27" s="104">
+      <c r="J27" s="105">
         <f>HYPERLINK("#'"&amp;"6. הודעות אחזקה (Notifications)"&amp;"'!A32","➜ פתח")</f>
         <v/>
       </c>
@@ -59947,12 +60091,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H28" s="54" t="inlineStr">
+      <c r="H28" s="106" t="inlineStr">
+        <is>
+          <t>QMEL.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I28" s="54" t="inlineStr">
         <is>
           <t>ההודעה מתייחסת לציוד</t>
         </is>
       </c>
-      <c r="I28" s="105">
+      <c r="J28" s="107">
         <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -59991,12 +60140,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H29" s="46" t="inlineStr">
+      <c r="H29" s="104" t="inlineStr">
+        <is>
+          <t>QMEL.TPLNR = IFLOT.TPLNR</t>
+        </is>
+      </c>
+      <c r="I29" s="46" t="inlineStr">
         <is>
           <t>ההודעה מתייחסת למיקום פונקציונלי</t>
         </is>
       </c>
-      <c r="I29" s="104">
+      <c r="J29" s="105">
         <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -60035,12 +60189,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H30" s="54" t="inlineStr">
+      <c r="H30" s="106" t="inlineStr">
+        <is>
+          <t>QMEL.OBJNR = JSTO.OBJNR</t>
+        </is>
+      </c>
+      <c r="I30" s="54" t="inlineStr">
         <is>
           <t>אובייקט הסטטוס של ההודעה</t>
         </is>
       </c>
-      <c r="I30" s="105">
+      <c r="J30" s="107">
         <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -60079,12 +60238,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H31" s="46" t="inlineStr">
+      <c r="H31" s="104" t="inlineStr">
+        <is>
+          <t>QMEL.QMART = TQ80.QMART</t>
+        </is>
+      </c>
+      <c r="I31" s="46" t="inlineStr">
         <is>
           <t>סוג ההודעה מגדיר פריסת מסך ופרופיל קטלוג</t>
         </is>
       </c>
-      <c r="I31" s="104">
+      <c r="J31" s="105">
         <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -60123,12 +60287,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H32" s="54" t="inlineStr">
+      <c r="H32" s="106" t="inlineStr">
+        <is>
+          <t>AFKO.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I32" s="54" t="inlineStr">
         <is>
           <t>כותרת נתוני האחזקה/ייצור של הפק"ע</t>
         </is>
       </c>
-      <c r="I32" s="105">
+      <c r="J32" s="107">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
@@ -60167,12 +60336,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H33" s="46" t="inlineStr">
+      <c r="H33" s="104" t="inlineStr">
+        <is>
+          <t>AFPO.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I33" s="46" t="inlineStr">
         <is>
           <t>פריטי הפק"ע</t>
         </is>
       </c>
-      <c r="I33" s="104">
+      <c r="J33" s="105">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
@@ -60211,12 +60385,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H34" s="54" t="inlineStr">
+      <c r="H34" s="106" t="inlineStr">
+        <is>
+          <t>AFIH.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I34" s="54" t="inlineStr">
         <is>
           <t>כותרת נתוני האחזקה (PM) של הפק"ע</t>
         </is>
       </c>
-      <c r="I34" s="105">
+      <c r="J34" s="107">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
         <v/>
       </c>
@@ -60255,12 +60434,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H35" s="46" t="inlineStr">
+      <c r="H35" s="104" t="inlineStr">
+        <is>
+          <t>AFVC.AUFPL = AFKO.AUFPL</t>
+        </is>
+      </c>
+      <c r="I35" s="46" t="inlineStr">
         <is>
           <t>פעולות הפק"ע תחת תוכנית הפעולות</t>
         </is>
       </c>
-      <c r="I35" s="104">
+      <c r="J35" s="105">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
@@ -60299,12 +60483,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H36" s="54" t="inlineStr">
+      <c r="H36" s="106" t="inlineStr">
+        <is>
+          <t>AFVC.ARBID = CRHD.OBJID</t>
+        </is>
+      </c>
+      <c r="I36" s="54" t="inlineStr">
         <is>
           <t>מרכז העבודה המבצע את הפעולה</t>
         </is>
       </c>
-      <c r="I36" s="105">
+      <c r="J36" s="107">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
@@ -60343,12 +60532,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H37" s="46" t="inlineStr">
+      <c r="H37" s="104" t="inlineStr">
+        <is>
+          <t>AFIH.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I37" s="46" t="inlineStr">
         <is>
           <t>הפק"ע מתייחסת לציוד</t>
         </is>
       </c>
-      <c r="I37" s="104">
+      <c r="J37" s="105">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
         <v/>
       </c>
@@ -60387,12 +60581,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H38" s="54" t="inlineStr">
+      <c r="H38" s="106" t="inlineStr">
+        <is>
+          <t>AFIH.TPLNR = IFLOT.TPLNR</t>
+        </is>
+      </c>
+      <c r="I38" s="54" t="inlineStr">
         <is>
           <t>הפק"ע מתייחסת למיקום פונקציונלי</t>
         </is>
       </c>
-      <c r="I38" s="105">
+      <c r="J38" s="107">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
         <v/>
       </c>
@@ -60431,12 +60630,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H39" s="46" t="inlineStr">
+      <c r="H39" s="104" t="inlineStr">
+        <is>
+          <t>AUFK.OBJNR = JSTO.OBJNR</t>
+        </is>
+      </c>
+      <c r="I39" s="46" t="inlineStr">
         <is>
           <t>אובייקט הסטטוס/CO של הפק"ע</t>
         </is>
       </c>
-      <c r="I39" s="104">
+      <c r="J39" s="105">
         <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
@@ -60475,12 +60679,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H40" s="54" t="inlineStr">
+      <c r="H40" s="106" t="inlineStr">
+        <is>
+          <t>AUFK.AUART = T003O.AUART</t>
+        </is>
+      </c>
+      <c r="I40" s="54" t="inlineStr">
         <is>
           <t>סוג הפקודה מגדיר פרמטרים, טווח מספרים ופרופיל סטטוס</t>
         </is>
       </c>
-      <c r="I40" s="105">
+      <c r="J40" s="107">
         <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
@@ -60519,12 +60728,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H41" s="46" t="inlineStr">
+      <c r="H41" s="104" t="inlineStr">
+        <is>
+          <t>JEST.OBJNR = JSTO.OBJNR</t>
+        </is>
+      </c>
+      <c r="I41" s="46" t="inlineStr">
         <is>
           <t>סטטוסים פעילים תחת אובייקט הסטטוס</t>
         </is>
       </c>
-      <c r="I41" s="104">
+      <c r="J41" s="105">
         <f>HYPERLINK("#'"&amp;"8. ניהול סטטוסים (Status Mgmt)"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -60563,12 +60777,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H42" s="54" t="inlineStr">
+      <c r="H42" s="106" t="inlineStr">
+        <is>
+          <t>JSTO.STSMA = TJ30.STSMA</t>
+        </is>
+      </c>
+      <c r="I42" s="54" t="inlineStr">
         <is>
           <t>פרופיל הסטטוס מגדיר את סטטוסי המשתמש</t>
         </is>
       </c>
-      <c r="I42" s="105">
+      <c r="J42" s="107">
         <f>HYPERLINK("#'"&amp;"8. ניהול סטטוסים (Status Mgmt)"&amp;"'!A9","➜ פתח")</f>
         <v/>
       </c>
@@ -60607,12 +60826,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H43" s="46" t="inlineStr">
+      <c r="H43" s="104" t="inlineStr">
+        <is>
+          <t>T003O.STSMA = TJ30.STSMA</t>
+        </is>
+      </c>
+      <c r="I43" s="46" t="inlineStr">
         <is>
           <t>פרופיל הסטטוס המשויך לסוג הפקודה</t>
         </is>
       </c>
-      <c r="I43" s="104">
+      <c r="J43" s="105">
         <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A45","➜ פתח")</f>
         <v/>
       </c>
@@ -60651,12 +60875,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H44" s="54" t="inlineStr">
+      <c r="H44" s="106" t="inlineStr">
+        <is>
+          <t>RESB.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I44" s="54" t="inlineStr">
         <is>
           <t>הזמנות רכיבים של הפק"ע</t>
         </is>
       </c>
-      <c r="I44" s="105">
+      <c r="J44" s="107">
         <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -60695,12 +60924,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H45" s="46" t="inlineStr">
+      <c r="H45" s="104" t="inlineStr">
+        <is>
+          <t>MSEG.MBLNR = MKPF.MBLNR</t>
+        </is>
+      </c>
+      <c r="I45" s="46" t="inlineStr">
         <is>
           <t>פריטי מסמך החומר תחת הכותרת</t>
         </is>
       </c>
-      <c r="I45" s="104">
+      <c r="J45" s="105">
         <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
@@ -60739,12 +60973,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H46" s="54" t="inlineStr">
+      <c r="H46" s="106" t="inlineStr">
+        <is>
+          <t>MSEG.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I46" s="54" t="inlineStr">
         <is>
           <t>תנועת המלאי מחויבת לפק"ע</t>
         </is>
       </c>
-      <c r="I46" s="105">
+      <c r="J46" s="107">
         <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
@@ -60783,12 +61022,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H47" s="46" t="inlineStr">
+      <c r="H47" s="104" t="inlineStr">
+        <is>
+          <t>EBKN.BANFN = EBAN.BANFN</t>
+        </is>
+      </c>
+      <c r="I47" s="46" t="inlineStr">
         <is>
           <t>חיוב דרישת הרכש</t>
         </is>
       </c>
-      <c r="I47" s="104">
+      <c r="J47" s="105">
         <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A18","➜ פתח")</f>
         <v/>
       </c>
@@ -60827,12 +61071,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H48" s="54" t="inlineStr">
+      <c r="H48" s="106" t="inlineStr">
+        <is>
+          <t>EBKN.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I48" s="54" t="inlineStr">
         <is>
           <t>דרישת הרכש מחויבת לפק"ע</t>
         </is>
       </c>
-      <c r="I48" s="105">
+      <c r="J48" s="107">
         <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A18","➜ פתח")</f>
         <v/>
       </c>
@@ -60871,12 +61120,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H49" s="46" t="inlineStr">
+      <c r="H49" s="104" t="inlineStr">
+        <is>
+          <t>COSP.OBJNR = AUFK.OBJNR</t>
+        </is>
+      </c>
+      <c r="I49" s="46" t="inlineStr">
         <is>
           <t>סך עלויות חיצוניות לפי אובייקט הפק"ע</t>
         </is>
       </c>
-      <c r="I49" s="104">
+      <c r="J49" s="105">
         <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
@@ -60915,12 +61169,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H50" s="54" t="inlineStr">
+      <c r="H50" s="106" t="inlineStr">
+        <is>
+          <t>COSS.OBJNR = AUFK.OBJNR</t>
+        </is>
+      </c>
+      <c r="I50" s="54" t="inlineStr">
         <is>
           <t>סך עלויות פנימיות לפי אובייקט הפק"ע</t>
         </is>
       </c>
-      <c r="I50" s="105">
+      <c r="J50" s="107">
         <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
@@ -60959,12 +61218,17 @@
           <t>1:1</t>
         </is>
       </c>
-      <c r="H51" s="46" t="inlineStr">
+      <c r="H51" s="104" t="inlineStr">
+        <is>
+          <t>COBRA.OBJNR = AUFK.OBJNR</t>
+        </is>
+      </c>
+      <c r="I51" s="46" t="inlineStr">
         <is>
           <t>כותרת חוק ההתחשבנות של הפק"ע</t>
         </is>
       </c>
-      <c r="I51" s="104">
+      <c r="J51" s="105">
         <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
@@ -61003,12 +61267,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H52" s="54" t="inlineStr">
+      <c r="H52" s="106" t="inlineStr">
+        <is>
+          <t>COBRB.OBJNR = COBRA.OBJNR</t>
+        </is>
+      </c>
+      <c r="I52" s="54" t="inlineStr">
         <is>
           <t>פריטי חוק ההתחשבנות (חוקי חלוקה)</t>
         </is>
       </c>
-      <c r="I52" s="105">
+      <c r="J52" s="107">
         <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A23","➜ פתח")</f>
         <v/>
       </c>
@@ -61047,12 +61316,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H53" s="46" t="inlineStr">
+      <c r="H53" s="104" t="inlineStr">
+        <is>
+          <t>MPOS.WARPL = MPLA.WARPL</t>
+        </is>
+      </c>
+      <c r="I53" s="46" t="inlineStr">
         <is>
           <t>פריטי תכנית האחזקה</t>
         </is>
       </c>
-      <c r="I53" s="104">
+      <c r="J53" s="105">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
@@ -61091,12 +61365,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H54" s="54" t="inlineStr">
+      <c r="H54" s="106" t="inlineStr">
+        <is>
+          <t>MPOS.EQUNR = EQUI.EQUNR</t>
+        </is>
+      </c>
+      <c r="I54" s="54" t="inlineStr">
         <is>
           <t>פריט התכנית מתייחס לציוד</t>
         </is>
       </c>
-      <c r="I54" s="105">
+      <c r="J54" s="107">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
@@ -61135,12 +61414,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H55" s="46" t="inlineStr">
+      <c r="H55" s="104" t="inlineStr">
+        <is>
+          <t>MPOS.PLNNR = PLKO.PLNNR</t>
+        </is>
+      </c>
+      <c r="I55" s="46" t="inlineStr">
         <is>
           <t>רשימת הפעולות המשויכת לפריט</t>
         </is>
       </c>
-      <c r="I55" s="104">
+      <c r="J55" s="105">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
@@ -61179,12 +61463,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H56" s="54" t="inlineStr">
+      <c r="H56" s="106" t="inlineStr">
+        <is>
+          <t>MHIO.WARPL = MPLA.WARPL</t>
+        </is>
+      </c>
+      <c r="I56" s="54" t="inlineStr">
         <is>
           <t>אובייקטי קריאת התכנית</t>
         </is>
       </c>
-      <c r="I56" s="105">
+      <c r="J56" s="107">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A33","➜ פתח")</f>
         <v/>
       </c>
@@ -61223,12 +61512,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H57" s="46" t="inlineStr">
+      <c r="H57" s="104" t="inlineStr">
+        <is>
+          <t>MHIO.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I57" s="46" t="inlineStr">
         <is>
           <t>הפק"ע שנוצרה מהקריאה</t>
         </is>
       </c>
-      <c r="I57" s="104">
+      <c r="J57" s="105">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A33","➜ פתח")</f>
         <v/>
       </c>
@@ -61267,12 +61561,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H58" s="54" t="inlineStr">
+      <c r="H58" s="106" t="inlineStr">
+        <is>
+          <t>MHIS.WARPL = MPLA.WARPL</t>
+        </is>
+      </c>
+      <c r="I58" s="54" t="inlineStr">
         <is>
           <t>היסטוריית התזמון של התכנית</t>
         </is>
       </c>
-      <c r="I58" s="105">
+      <c r="J58" s="107">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A40","➜ פתח")</f>
         <v/>
       </c>
@@ -61311,12 +61610,17 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H59" s="46" t="inlineStr">
+      <c r="H59" s="104" t="inlineStr">
+        <is>
+          <t>PLPO.PLNNR = PLKO.PLNNR</t>
+        </is>
+      </c>
+      <c r="I59" s="46" t="inlineStr">
         <is>
           <t>פעולות רשימת הפעולות תחת הכותרת</t>
         </is>
       </c>
-      <c r="I59" s="104">
+      <c r="J59" s="105">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
@@ -61355,19 +61659,24 @@
           <t>N:1</t>
         </is>
       </c>
-      <c r="H60" s="54" t="inlineStr">
+      <c r="H60" s="106" t="inlineStr">
+        <is>
+          <t>PLPO.ARBID = CRHD.OBJID</t>
+        </is>
+      </c>
+      <c r="I60" s="54" t="inlineStr">
         <is>
           <t>מרכז העבודה של הפעולה ברשימה</t>
         </is>
       </c>
-      <c r="I60" s="105">
+      <c r="J60" s="107">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="C1:J1"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <hyperlinks>

</xml_diff>

<commit_message>
Final production build: complete JOIN ON coverage for config tables (TQ80/T003O/TJ30/BUT000 via CVI); full hyperlink + back-button integrity validated
</commit_message>
<xml_diff>
--- a/SAP_PM_ECC6_to_S4_Migration.xlsx
+++ b/SAP_PM_ECC6_to_S4_Migration.xlsx
@@ -58,7 +58,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="15">'Custom Code Check'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="15">'Custom Code Check'!$A$1:$I$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="16">'ER - Join Map'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="16">'ER - Join Map'!$A$1:$J$60</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="16">'ER - Join Map'!$A$1:$J$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1358,7 +1358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V906"/>
+  <dimension ref="A1:V909"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2929,7 +2929,7 @@
     <row r="28">
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="33">
-        <f>IF(C25="","הקלד מונח בתא הצהוב למעלה - והתוצאות יופיעו כאן מיד (כולל קישור לחיץ)...",IFERROR(_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6},$V$2:$V$906,$Q$2:$Q$906,$R$2:$R$906,$S$2:$S$906,$T$2:$T$906,$U$2:$U$906),(ISNUMBER(SEARCH(C25,$Q$2:$Q$906)))+(ISNUMBER(SEARCH(C25,$R$2:$R$906)))+(ISNUMBER(SEARCH(C25,$S$2:$S$906)))+(ISNUMBER(SEARCH(C25,$P$2:$P$906)))&gt;0),"לא נמצאו תוצאות - נסה מונח אחר"))</f>
+        <f>IF(C25="","הקלד מונח בתא הצהוב למעלה - והתוצאות יופיעו כאן מיד (כולל קישור לחיץ)...",IFERROR(_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6},$V$2:$V$909,$Q$2:$Q$909,$R$2:$R$909,$S$2:$S$909,$T$2:$T$909,$U$2:$U$909),(ISNUMBER(SEARCH(C25,$Q$2:$Q$909)))+(ISNUMBER(SEARCH(C25,$R$2:$R$909)))+(ISNUMBER(SEARCH(C25,$S$2:$S$909)))+(ISNUMBER(SEARCH(C25,$P$2:$P$909)))&gt;0),"לא נמצאו תוצאות - נסה מונח אחר"))</f>
         <v/>
       </c>
       <c r="C28" s="1" t="n"/>
@@ -46006,12 +46006,12 @@
       </c>
       <c r="Q878" s="8" t="inlineStr">
         <is>
-          <t>AFKO.AUFNR = AUFK.AUFNR</t>
+          <t>TQ80.RBNR = T352.RBNR</t>
         </is>
       </c>
       <c r="R878" s="7" t="inlineStr">
         <is>
-          <t>כותרת נתוני האחזקה/ייצור של הפק"ע</t>
+          <t>סוג ההודעה מפנה לפרופיל הקטלוג (קודים מותרים)</t>
         </is>
       </c>
       <c r="S878" s="7" t="inlineStr"/>
@@ -46053,12 +46053,12 @@
       </c>
       <c r="Q879" s="8" t="inlineStr">
         <is>
-          <t>AFPO.AUFNR = AUFK.AUFNR</t>
+          <t>TQ80.AUART = T003O.AUART</t>
         </is>
       </c>
       <c r="R879" s="7" t="inlineStr">
         <is>
-          <t>פריטי הפק"ע</t>
+          <t>סוג ההודעה מגדיר סוג פק"ע ברירת מחדל</t>
         </is>
       </c>
       <c r="S879" s="7" t="inlineStr"/>
@@ -46100,12 +46100,12 @@
       </c>
       <c r="Q880" s="8" t="inlineStr">
         <is>
-          <t>AFIH.AUFNR = AUFK.AUFNR</t>
+          <t>AFKO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R880" s="7" t="inlineStr">
         <is>
-          <t>כותרת נתוני האחזקה (PM) של הפק"ע</t>
+          <t>כותרת נתוני האחזקה/ייצור של הפק"ע</t>
         </is>
       </c>
       <c r="S880" s="7" t="inlineStr"/>
@@ -46147,12 +46147,12 @@
       </c>
       <c r="Q881" s="8" t="inlineStr">
         <is>
-          <t>AFVC.AUFPL = AFKO.AUFPL</t>
+          <t>AFPO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R881" s="7" t="inlineStr">
         <is>
-          <t>פעולות הפק"ע תחת תוכנית הפעולות</t>
+          <t>פריטי הפק"ע</t>
         </is>
       </c>
       <c r="S881" s="7" t="inlineStr"/>
@@ -46194,12 +46194,12 @@
       </c>
       <c r="Q882" s="8" t="inlineStr">
         <is>
-          <t>AFVC.ARBID = CRHD.OBJID</t>
+          <t>AFIH.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R882" s="7" t="inlineStr">
         <is>
-          <t>מרכז העבודה המבצע את הפעולה</t>
+          <t>כותרת נתוני האחזקה (PM) של הפק"ע</t>
         </is>
       </c>
       <c r="S882" s="7" t="inlineStr"/>
@@ -46241,12 +46241,12 @@
       </c>
       <c r="Q883" s="8" t="inlineStr">
         <is>
-          <t>AFIH.EQUNR = EQUI.EQUNR</t>
+          <t>AFVC.AUFPL = AFKO.AUFPL</t>
         </is>
       </c>
       <c r="R883" s="7" t="inlineStr">
         <is>
-          <t>הפק"ע מתייחסת לציוד</t>
+          <t>פעולות הפק"ע תחת תוכנית הפעולות</t>
         </is>
       </c>
       <c r="S883" s="7" t="inlineStr"/>
@@ -46288,12 +46288,12 @@
       </c>
       <c r="Q884" s="8" t="inlineStr">
         <is>
-          <t>AFIH.TPLNR = IFLOT.TPLNR</t>
+          <t>AFVC.ARBID = CRHD.OBJID</t>
         </is>
       </c>
       <c r="R884" s="7" t="inlineStr">
         <is>
-          <t>הפק"ע מתייחסת למיקום פונקציונלי</t>
+          <t>מרכז העבודה המבצע את הפעולה</t>
         </is>
       </c>
       <c r="S884" s="7" t="inlineStr"/>
@@ -46335,12 +46335,12 @@
       </c>
       <c r="Q885" s="8" t="inlineStr">
         <is>
-          <t>AUFK.OBJNR = JSTO.OBJNR</t>
+          <t>AFIH.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R885" s="7" t="inlineStr">
         <is>
-          <t>אובייקט הסטטוס/CO של הפק"ע</t>
+          <t>הפק"ע מתייחסת לציוד</t>
         </is>
       </c>
       <c r="S885" s="7" t="inlineStr"/>
@@ -46382,12 +46382,12 @@
       </c>
       <c r="Q886" s="8" t="inlineStr">
         <is>
-          <t>AUFK.AUART = T003O.AUART</t>
+          <t>AFIH.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="R886" s="7" t="inlineStr">
         <is>
-          <t>סוג הפקודה מגדיר פרמטרים, טווח מספרים ופרופיל סטטוס</t>
+          <t>הפק"ע מתייחסת למיקום פונקציונלי</t>
         </is>
       </c>
       <c r="S886" s="7" t="inlineStr"/>
@@ -46429,12 +46429,12 @@
       </c>
       <c r="Q887" s="8" t="inlineStr">
         <is>
-          <t>JEST.OBJNR = JSTO.OBJNR</t>
+          <t>AUFK.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R887" s="7" t="inlineStr">
         <is>
-          <t>סטטוסים פעילים תחת אובייקט הסטטוס</t>
+          <t>אובייקט הסטטוס/CO של הפק"ע</t>
         </is>
       </c>
       <c r="S887" s="7" t="inlineStr"/>
@@ -46476,12 +46476,12 @@
       </c>
       <c r="Q888" s="8" t="inlineStr">
         <is>
-          <t>JSTO.STSMA = TJ30.STSMA</t>
+          <t>AUFK.AUART = T003O.AUART</t>
         </is>
       </c>
       <c r="R888" s="7" t="inlineStr">
         <is>
-          <t>פרופיל הסטטוס מגדיר את סטטוסי המשתמש</t>
+          <t>סוג הפקודה מגדיר פרמטרים, טווח מספרים ופרופיל סטטוס</t>
         </is>
       </c>
       <c r="S888" s="7" t="inlineStr"/>
@@ -46523,12 +46523,12 @@
       </c>
       <c r="Q889" s="8" t="inlineStr">
         <is>
-          <t>T003O.STSMA = TJ30.STSMA</t>
+          <t>JEST.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="R889" s="7" t="inlineStr">
         <is>
-          <t>פרופיל הסטטוס המשויך לסוג הפקודה</t>
+          <t>סטטוסים פעילים תחת אובייקט הסטטוס</t>
         </is>
       </c>
       <c r="S889" s="7" t="inlineStr"/>
@@ -46570,12 +46570,12 @@
       </c>
       <c r="Q890" s="8" t="inlineStr">
         <is>
-          <t>RESB.AUFNR = AUFK.AUFNR</t>
+          <t>JSTO.STSMA = TJ30.STSMA</t>
         </is>
       </c>
       <c r="R890" s="7" t="inlineStr">
         <is>
-          <t>הזמנות רכיבים של הפק"ע</t>
+          <t>פרופיל הסטטוס מגדיר את סטטוסי המשתמש</t>
         </is>
       </c>
       <c r="S890" s="7" t="inlineStr"/>
@@ -46617,12 +46617,12 @@
       </c>
       <c r="Q891" s="8" t="inlineStr">
         <is>
-          <t>MSEG.MBLNR = MKPF.MBLNR</t>
+          <t>T003O.STSMA = TJ30.STSMA</t>
         </is>
       </c>
       <c r="R891" s="7" t="inlineStr">
         <is>
-          <t>פריטי מסמך החומר תחת הכותרת</t>
+          <t>פרופיל הסטטוס המשויך לסוג הפקודה</t>
         </is>
       </c>
       <c r="S891" s="7" t="inlineStr"/>
@@ -46664,12 +46664,12 @@
       </c>
       <c r="Q892" s="8" t="inlineStr">
         <is>
-          <t>MSEG.AUFNR = AUFK.AUFNR</t>
+          <t>RESB.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R892" s="7" t="inlineStr">
         <is>
-          <t>תנועת המלאי מחויבת לפק"ע</t>
+          <t>הזמנות רכיבים של הפק"ע</t>
         </is>
       </c>
       <c r="S892" s="7" t="inlineStr"/>
@@ -46711,12 +46711,12 @@
       </c>
       <c r="Q893" s="8" t="inlineStr">
         <is>
-          <t>EBKN.BANFN = EBAN.BANFN</t>
+          <t>MSEG.MBLNR = MKPF.MBLNR</t>
         </is>
       </c>
       <c r="R893" s="7" t="inlineStr">
         <is>
-          <t>חיוב דרישת הרכש</t>
+          <t>פריטי מסמך החומר תחת הכותרת</t>
         </is>
       </c>
       <c r="S893" s="7" t="inlineStr"/>
@@ -46758,12 +46758,12 @@
       </c>
       <c r="Q894" s="8" t="inlineStr">
         <is>
-          <t>EBKN.AUFNR = AUFK.AUFNR</t>
+          <t>MSEG.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R894" s="7" t="inlineStr">
         <is>
-          <t>דרישת הרכש מחויבת לפק"ע</t>
+          <t>תנועת המלאי מחויבת לפק"ע</t>
         </is>
       </c>
       <c r="S894" s="7" t="inlineStr"/>
@@ -46805,12 +46805,12 @@
       </c>
       <c r="Q895" s="8" t="inlineStr">
         <is>
-          <t>COSP.OBJNR = AUFK.OBJNR</t>
+          <t>EBKN.BANFN = EBAN.BANFN</t>
         </is>
       </c>
       <c r="R895" s="7" t="inlineStr">
         <is>
-          <t>סך עלויות חיצוניות לפי אובייקט הפק"ע</t>
+          <t>חיוב דרישת הרכש</t>
         </is>
       </c>
       <c r="S895" s="7" t="inlineStr"/>
@@ -46852,12 +46852,12 @@
       </c>
       <c r="Q896" s="8" t="inlineStr">
         <is>
-          <t>COSS.OBJNR = AUFK.OBJNR</t>
+          <t>EBKN.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R896" s="7" t="inlineStr">
         <is>
-          <t>סך עלויות פנימיות לפי אובייקט הפק"ע</t>
+          <t>דרישת הרכש מחויבת לפק"ע</t>
         </is>
       </c>
       <c r="S896" s="7" t="inlineStr"/>
@@ -46899,12 +46899,12 @@
       </c>
       <c r="Q897" s="8" t="inlineStr">
         <is>
-          <t>COBRA.OBJNR = AUFK.OBJNR</t>
+          <t>EBAN.FLIEF = BUT000.PARTNER</t>
         </is>
       </c>
       <c r="R897" s="7" t="inlineStr">
         <is>
-          <t>כותרת חוק ההתחשבנות של הפק"ע</t>
+          <t>ספק קבוע בדרישת הרכש - ב-S/4 דרך Business Partner (CVI)</t>
         </is>
       </c>
       <c r="S897" s="7" t="inlineStr"/>
@@ -46946,12 +46946,12 @@
       </c>
       <c r="Q898" s="8" t="inlineStr">
         <is>
-          <t>COBRB.OBJNR = COBRA.OBJNR</t>
+          <t>COSP.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="R898" s="7" t="inlineStr">
         <is>
-          <t>פריטי חוק ההתחשבנות (חוקי חלוקה)</t>
+          <t>סך עלויות חיצוניות לפי אובייקט הפק"ע</t>
         </is>
       </c>
       <c r="S898" s="7" t="inlineStr"/>
@@ -46993,12 +46993,12 @@
       </c>
       <c r="Q899" s="8" t="inlineStr">
         <is>
-          <t>MPOS.WARPL = MPLA.WARPL</t>
+          <t>COSS.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="R899" s="7" t="inlineStr">
         <is>
-          <t>פריטי תכנית האחזקה</t>
+          <t>סך עלויות פנימיות לפי אובייקט הפק"ע</t>
         </is>
       </c>
       <c r="S899" s="7" t="inlineStr"/>
@@ -47040,12 +47040,12 @@
       </c>
       <c r="Q900" s="8" t="inlineStr">
         <is>
-          <t>MPOS.EQUNR = EQUI.EQUNR</t>
+          <t>COBRA.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="R900" s="7" t="inlineStr">
         <is>
-          <t>פריט התכנית מתייחס לציוד</t>
+          <t>כותרת חוק ההתחשבנות של הפק"ע</t>
         </is>
       </c>
       <c r="S900" s="7" t="inlineStr"/>
@@ -47087,12 +47087,12 @@
       </c>
       <c r="Q901" s="8" t="inlineStr">
         <is>
-          <t>MPOS.PLNNR = PLKO.PLNNR</t>
+          <t>COBRB.OBJNR = COBRA.OBJNR</t>
         </is>
       </c>
       <c r="R901" s="7" t="inlineStr">
         <is>
-          <t>רשימת הפעולות המשויכת לפריט</t>
+          <t>פריטי חוק ההתחשבנות (חוקי חלוקה)</t>
         </is>
       </c>
       <c r="S901" s="7" t="inlineStr"/>
@@ -47134,12 +47134,12 @@
       </c>
       <c r="Q902" s="8" t="inlineStr">
         <is>
-          <t>MHIO.WARPL = MPLA.WARPL</t>
+          <t>MPOS.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="R902" s="7" t="inlineStr">
         <is>
-          <t>אובייקטי קריאת התכנית</t>
+          <t>פריטי תכנית האחזקה</t>
         </is>
       </c>
       <c r="S902" s="7" t="inlineStr"/>
@@ -47181,12 +47181,12 @@
       </c>
       <c r="Q903" s="8" t="inlineStr">
         <is>
-          <t>MHIO.AUFNR = AUFK.AUFNR</t>
+          <t>MPOS.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="R903" s="7" t="inlineStr">
         <is>
-          <t>הפק"ע שנוצרה מהקריאה</t>
+          <t>פריט התכנית מתייחס לציוד</t>
         </is>
       </c>
       <c r="S903" s="7" t="inlineStr"/>
@@ -47228,12 +47228,12 @@
       </c>
       <c r="Q904" s="8" t="inlineStr">
         <is>
-          <t>MHIS.WARPL = MPLA.WARPL</t>
+          <t>MPOS.PLNNR = PLKO.PLNNR</t>
         </is>
       </c>
       <c r="R904" s="7" t="inlineStr">
         <is>
-          <t>היסטוריית התזמון של התכנית</t>
+          <t>רשימת הפעולות המשויכת לפריט</t>
         </is>
       </c>
       <c r="S904" s="7" t="inlineStr"/>
@@ -47275,12 +47275,12 @@
       </c>
       <c r="Q905" s="8" t="inlineStr">
         <is>
-          <t>PLPO.PLNNR = PLKO.PLNNR</t>
+          <t>MHIO.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="R905" s="7" t="inlineStr">
         <is>
-          <t>פעולות רשימת הפעולות תחת הכותרת</t>
+          <t>אובייקטי קריאת התכנית</t>
         </is>
       </c>
       <c r="S905" s="7" t="inlineStr"/>
@@ -47322,12 +47322,12 @@
       </c>
       <c r="Q906" s="8" t="inlineStr">
         <is>
-          <t>PLPO.ARBID = CRHD.OBJID</t>
+          <t>MHIO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="R906" s="7" t="inlineStr">
         <is>
-          <t>מרכז העבודה של הפעולה ברשימה</t>
+          <t>הפק"ע שנוצרה מהקריאה</t>
         </is>
       </c>
       <c r="S906" s="7" t="inlineStr"/>
@@ -47343,6 +47343,147 @@
       </c>
       <c r="V906" s="9">
         <f>HYPERLINK("#'"&amp;T906&amp;"'!"&amp;U906,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="4" t="n"/>
+      <c r="B907" s="4" t="n"/>
+      <c r="C907" s="4" t="n"/>
+      <c r="D907" s="4" t="n"/>
+      <c r="E907" s="4" t="n"/>
+      <c r="F907" s="4" t="n"/>
+      <c r="G907" s="4" t="n"/>
+      <c r="H907" s="4" t="n"/>
+      <c r="I907" s="4" t="n"/>
+      <c r="J907" s="4" t="n"/>
+      <c r="K907" s="4" t="n"/>
+      <c r="L907" s="4" t="n"/>
+      <c r="M907" s="4" t="n"/>
+      <c r="N907" s="4" t="n"/>
+      <c r="O907" s="4" t="n"/>
+      <c r="P907" s="7" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="Q907" s="8" t="inlineStr">
+        <is>
+          <t>MHIS.WARPL = MPLA.WARPL</t>
+        </is>
+      </c>
+      <c r="R907" s="7" t="inlineStr">
+        <is>
+          <t>היסטוריית התזמון של התכנית</t>
+        </is>
+      </c>
+      <c r="S907" s="7" t="inlineStr"/>
+      <c r="T907" s="7" t="inlineStr">
+        <is>
+          <t>ER - Join Map</t>
+        </is>
+      </c>
+      <c r="U907" s="7" t="inlineStr">
+        <is>
+          <t>A61</t>
+        </is>
+      </c>
+      <c r="V907" s="9">
+        <f>HYPERLINK("#'"&amp;T907&amp;"'!"&amp;U907,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="4" t="n"/>
+      <c r="B908" s="4" t="n"/>
+      <c r="C908" s="4" t="n"/>
+      <c r="D908" s="4" t="n"/>
+      <c r="E908" s="4" t="n"/>
+      <c r="F908" s="4" t="n"/>
+      <c r="G908" s="4" t="n"/>
+      <c r="H908" s="4" t="n"/>
+      <c r="I908" s="4" t="n"/>
+      <c r="J908" s="4" t="n"/>
+      <c r="K908" s="4" t="n"/>
+      <c r="L908" s="4" t="n"/>
+      <c r="M908" s="4" t="n"/>
+      <c r="N908" s="4" t="n"/>
+      <c r="O908" s="4" t="n"/>
+      <c r="P908" s="7" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="Q908" s="8" t="inlineStr">
+        <is>
+          <t>PLPO.PLNNR = PLKO.PLNNR</t>
+        </is>
+      </c>
+      <c r="R908" s="7" t="inlineStr">
+        <is>
+          <t>פעולות רשימת הפעולות תחת הכותרת</t>
+        </is>
+      </c>
+      <c r="S908" s="7" t="inlineStr"/>
+      <c r="T908" s="7" t="inlineStr">
+        <is>
+          <t>ER - Join Map</t>
+        </is>
+      </c>
+      <c r="U908" s="7" t="inlineStr">
+        <is>
+          <t>A62</t>
+        </is>
+      </c>
+      <c r="V908" s="9">
+        <f>HYPERLINK("#'"&amp;T908&amp;"'!"&amp;U908,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="4" t="n"/>
+      <c r="B909" s="4" t="n"/>
+      <c r="C909" s="4" t="n"/>
+      <c r="D909" s="4" t="n"/>
+      <c r="E909" s="4" t="n"/>
+      <c r="F909" s="4" t="n"/>
+      <c r="G909" s="4" t="n"/>
+      <c r="H909" s="4" t="n"/>
+      <c r="I909" s="4" t="n"/>
+      <c r="J909" s="4" t="n"/>
+      <c r="K909" s="4" t="n"/>
+      <c r="L909" s="4" t="n"/>
+      <c r="M909" s="4" t="n"/>
+      <c r="N909" s="4" t="n"/>
+      <c r="O909" s="4" t="n"/>
+      <c r="P909" s="7" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="Q909" s="8" t="inlineStr">
+        <is>
+          <t>PLPO.ARBID = CRHD.OBJID</t>
+        </is>
+      </c>
+      <c r="R909" s="7" t="inlineStr">
+        <is>
+          <t>מרכז העבודה של הפעולה ברשימה</t>
+        </is>
+      </c>
+      <c r="S909" s="7" t="inlineStr"/>
+      <c r="T909" s="7" t="inlineStr">
+        <is>
+          <t>ER - Join Map</t>
+        </is>
+      </c>
+      <c r="U909" s="7" t="inlineStr">
+        <is>
+          <t>A63</t>
+        </is>
+      </c>
+      <c r="V909" s="9">
+        <f>HYPERLINK("#'"&amp;T909&amp;"'!"&amp;U909,"➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -58745,7 +58886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -60259,12 +60400,12 @@
       </c>
       <c r="B32" s="103" t="inlineStr">
         <is>
-          <t>AFKO</t>
+          <t>TQ80</t>
         </is>
       </c>
       <c r="C32" s="103" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>RBNR</t>
         </is>
       </c>
       <c r="D32" s="100" t="inlineStr">
@@ -60274,31 +60415,31 @@
       </c>
       <c r="E32" s="52" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>T352</t>
         </is>
       </c>
       <c r="F32" s="52" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>RBNR</t>
         </is>
       </c>
       <c r="G32" s="100" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>N:1</t>
         </is>
       </c>
       <c r="H32" s="106" t="inlineStr">
         <is>
-          <t>AFKO.AUFNR = AUFK.AUFNR</t>
+          <t>TQ80.RBNR = T352.RBNR</t>
         </is>
       </c>
       <c r="I32" s="54" t="inlineStr">
         <is>
-          <t>כותרת נתוני האחזקה/ייצור של הפק"ע</t>
+          <t>סוג ההודעה מפנה לפרופיל הקטלוג (קודים מותרים)</t>
         </is>
       </c>
       <c r="J32" s="107">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A10","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"6. הודעות אחזקה (Notifications)"&amp;"'!A39","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60308,12 +60449,12 @@
       </c>
       <c r="B33" s="102" t="inlineStr">
         <is>
-          <t>AFPO</t>
+          <t>TQ80</t>
         </is>
       </c>
       <c r="C33" s="102" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>AUART</t>
         </is>
       </c>
       <c r="D33" s="96" t="inlineStr">
@@ -60323,12 +60464,12 @@
       </c>
       <c r="E33" s="44" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>T003O</t>
         </is>
       </c>
       <c r="F33" s="44" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>AUART</t>
         </is>
       </c>
       <c r="G33" s="96" t="inlineStr">
@@ -60338,16 +60479,16 @@
       </c>
       <c r="H33" s="104" t="inlineStr">
         <is>
-          <t>AFPO.AUFNR = AUFK.AUFNR</t>
+          <t>TQ80.AUART = T003O.AUART</t>
         </is>
       </c>
       <c r="I33" s="46" t="inlineStr">
         <is>
-          <t>פריטי הפק"ע</t>
+          <t>סוג ההודעה מגדיר סוג פק"ע ברירת מחדל</t>
         </is>
       </c>
       <c r="J33" s="105">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A25","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"6. הודעות אחזקה (Notifications)"&amp;"'!A39","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60357,7 +60498,7 @@
       </c>
       <c r="B34" s="103" t="inlineStr">
         <is>
-          <t>AFIH</t>
+          <t>AFKO</t>
         </is>
       </c>
       <c r="C34" s="103" t="inlineStr">
@@ -60387,16 +60528,16 @@
       </c>
       <c r="H34" s="106" t="inlineStr">
         <is>
-          <t>AFIH.AUFNR = AUFK.AUFNR</t>
+          <t>AFKO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="I34" s="54" t="inlineStr">
         <is>
-          <t>כותרת נתוני האחזקה (PM) של הפק"ע</t>
+          <t>כותרת נתוני האחזקה/ייצור של הפק"ע</t>
         </is>
       </c>
       <c r="J34" s="107">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60406,12 +60547,12 @@
       </c>
       <c r="B35" s="102" t="inlineStr">
         <is>
-          <t>AFVC</t>
+          <t>AFPO</t>
         </is>
       </c>
       <c r="C35" s="102" t="inlineStr">
         <is>
-          <t>AUFPL</t>
+          <t>AUFNR</t>
         </is>
       </c>
       <c r="D35" s="96" t="inlineStr">
@@ -60421,12 +60562,12 @@
       </c>
       <c r="E35" s="44" t="inlineStr">
         <is>
-          <t>AFKO</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="F35" s="44" t="inlineStr">
         <is>
-          <t>AUFPL</t>
+          <t>AUFNR</t>
         </is>
       </c>
       <c r="G35" s="96" t="inlineStr">
@@ -60436,16 +60577,16 @@
       </c>
       <c r="H35" s="104" t="inlineStr">
         <is>
-          <t>AFVC.AUFPL = AFKO.AUFPL</t>
+          <t>AFPO.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="I35" s="46" t="inlineStr">
         <is>
-          <t>פעולות הפק"ע תחת תוכנית הפעולות</t>
+          <t>פריטי הפק"ע</t>
         </is>
       </c>
       <c r="J35" s="105">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A17","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60455,12 +60596,12 @@
       </c>
       <c r="B36" s="103" t="inlineStr">
         <is>
-          <t>AFVC</t>
+          <t>AFIH</t>
         </is>
       </c>
       <c r="C36" s="103" t="inlineStr">
         <is>
-          <t>ARBID</t>
+          <t>AUFNR</t>
         </is>
       </c>
       <c r="D36" s="100" t="inlineStr">
@@ -60470,31 +60611,31 @@
       </c>
       <c r="E36" s="52" t="inlineStr">
         <is>
-          <t>CRHD</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="F36" s="52" t="inlineStr">
         <is>
-          <t>OBJID</t>
+          <t>AUFNR</t>
         </is>
       </c>
       <c r="G36" s="100" t="inlineStr">
         <is>
-          <t>N:1</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="H36" s="106" t="inlineStr">
         <is>
-          <t>AFVC.ARBID = CRHD.OBJID</t>
+          <t>AFIH.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="I36" s="54" t="inlineStr">
         <is>
-          <t>מרכז העבודה המבצע את הפעולה</t>
+          <t>כותרת נתוני האחזקה (PM) של הפק"ע</t>
         </is>
       </c>
       <c r="J36" s="107">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A17","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60504,12 +60645,12 @@
       </c>
       <c r="B37" s="102" t="inlineStr">
         <is>
-          <t>AFIH</t>
+          <t>AFVC</t>
         </is>
       </c>
       <c r="C37" s="102" t="inlineStr">
         <is>
-          <t>EQUNR</t>
+          <t>AUFPL</t>
         </is>
       </c>
       <c r="D37" s="96" t="inlineStr">
@@ -60519,12 +60660,12 @@
       </c>
       <c r="E37" s="44" t="inlineStr">
         <is>
-          <t>EQUI</t>
+          <t>AFKO</t>
         </is>
       </c>
       <c r="F37" s="44" t="inlineStr">
         <is>
-          <t>EQUNR</t>
+          <t>AUFPL</t>
         </is>
       </c>
       <c r="G37" s="96" t="inlineStr">
@@ -60534,16 +60675,16 @@
       </c>
       <c r="H37" s="104" t="inlineStr">
         <is>
-          <t>AFIH.EQUNR = EQUI.EQUNR</t>
+          <t>AFVC.AUFPL = AFKO.AUFPL</t>
         </is>
       </c>
       <c r="I37" s="46" t="inlineStr">
         <is>
-          <t>הפק"ע מתייחסת לציוד</t>
+          <t>פעולות הפק"ע תחת תוכנית הפעולות</t>
         </is>
       </c>
       <c r="J37" s="105">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60553,12 +60694,12 @@
       </c>
       <c r="B38" s="103" t="inlineStr">
         <is>
-          <t>AFIH</t>
+          <t>AFVC</t>
         </is>
       </c>
       <c r="C38" s="103" t="inlineStr">
         <is>
-          <t>TPLNR</t>
+          <t>ARBID</t>
         </is>
       </c>
       <c r="D38" s="100" t="inlineStr">
@@ -60568,12 +60709,12 @@
       </c>
       <c r="E38" s="52" t="inlineStr">
         <is>
-          <t>IFLOT</t>
+          <t>CRHD</t>
         </is>
       </c>
       <c r="F38" s="52" t="inlineStr">
         <is>
-          <t>TPLNR</t>
+          <t>OBJID</t>
         </is>
       </c>
       <c r="G38" s="100" t="inlineStr">
@@ -60583,16 +60724,16 @@
       </c>
       <c r="H38" s="106" t="inlineStr">
         <is>
-          <t>AFIH.TPLNR = IFLOT.TPLNR</t>
+          <t>AFVC.ARBID = CRHD.OBJID</t>
         </is>
       </c>
       <c r="I38" s="54" t="inlineStr">
         <is>
-          <t>הפק"ע מתייחסת למיקום פונקציונלי</t>
+          <t>מרכז העבודה המבצע את הפעולה</t>
         </is>
       </c>
       <c r="J38" s="107">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60602,12 +60743,12 @@
       </c>
       <c r="B39" s="102" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>AFIH</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>EQUNR</t>
         </is>
       </c>
       <c r="D39" s="96" t="inlineStr">
@@ -60617,31 +60758,31 @@
       </c>
       <c r="E39" s="44" t="inlineStr">
         <is>
-          <t>JSTO</t>
+          <t>EQUI</t>
         </is>
       </c>
       <c r="F39" s="44" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>EQUNR</t>
         </is>
       </c>
       <c r="G39" s="96" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>N:1</t>
         </is>
       </c>
       <c r="H39" s="104" t="inlineStr">
         <is>
-          <t>AUFK.OBJNR = JSTO.OBJNR</t>
+          <t>AFIH.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="I39" s="46" t="inlineStr">
         <is>
-          <t>אובייקט הסטטוס/CO של הפק"ע</t>
+          <t>הפק"ע מתייחסת לציוד</t>
         </is>
       </c>
       <c r="J39" s="105">
-        <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A10","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60651,12 +60792,12 @@
       </c>
       <c r="B40" s="103" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>AFIH</t>
         </is>
       </c>
       <c r="C40" s="103" t="inlineStr">
         <is>
-          <t>AUART</t>
+          <t>TPLNR</t>
         </is>
       </c>
       <c r="D40" s="100" t="inlineStr">
@@ -60666,12 +60807,12 @@
       </c>
       <c r="E40" s="52" t="inlineStr">
         <is>
-          <t>T003O</t>
+          <t>IFLOT</t>
         </is>
       </c>
       <c r="F40" s="52" t="inlineStr">
         <is>
-          <t>AUART</t>
+          <t>TPLNR</t>
         </is>
       </c>
       <c r="G40" s="100" t="inlineStr">
@@ -60681,16 +60822,16 @@
       </c>
       <c r="H40" s="106" t="inlineStr">
         <is>
-          <t>AUFK.AUART = T003O.AUART</t>
+          <t>AFIH.TPLNR = IFLOT.TPLNR</t>
         </is>
       </c>
       <c r="I40" s="54" t="inlineStr">
         <is>
-          <t>סוג הפקודה מגדיר פרמטרים, טווח מספרים ופרופיל סטטוס</t>
+          <t>הפק"ע מתייחסת למיקום פונקציונלי</t>
         </is>
       </c>
       <c r="J40" s="107">
-        <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A10","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A31","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60700,7 +60841,7 @@
       </c>
       <c r="B41" s="102" t="inlineStr">
         <is>
-          <t>JEST</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="C41" s="102" t="inlineStr">
@@ -60725,21 +60866,21 @@
       </c>
       <c r="G41" s="96" t="inlineStr">
         <is>
-          <t>N:1</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="H41" s="104" t="inlineStr">
         <is>
-          <t>JEST.OBJNR = JSTO.OBJNR</t>
+          <t>AUFK.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="I41" s="46" t="inlineStr">
         <is>
-          <t>סטטוסים פעילים תחת אובייקט הסטטוס</t>
+          <t>אובייקט הסטטוס/CO של הפק"ע</t>
         </is>
       </c>
       <c r="J41" s="105">
-        <f>HYPERLINK("#'"&amp;"8. ניהול סטטוסים (Status Mgmt)"&amp;"'!A3","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60749,12 +60890,12 @@
       </c>
       <c r="B42" s="103" t="inlineStr">
         <is>
-          <t>JSTO</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="C42" s="103" t="inlineStr">
         <is>
-          <t>STSMA</t>
+          <t>AUART</t>
         </is>
       </c>
       <c r="D42" s="100" t="inlineStr">
@@ -60764,12 +60905,12 @@
       </c>
       <c r="E42" s="52" t="inlineStr">
         <is>
-          <t>TJ30</t>
+          <t>T003O</t>
         </is>
       </c>
       <c r="F42" s="52" t="inlineStr">
         <is>
-          <t>STSMA</t>
+          <t>AUART</t>
         </is>
       </c>
       <c r="G42" s="100" t="inlineStr">
@@ -60779,16 +60920,16 @@
       </c>
       <c r="H42" s="106" t="inlineStr">
         <is>
-          <t>JSTO.STSMA = TJ30.STSMA</t>
+          <t>AUFK.AUART = T003O.AUART</t>
         </is>
       </c>
       <c r="I42" s="54" t="inlineStr">
         <is>
-          <t>פרופיל הסטטוס מגדיר את סטטוסי המשתמש</t>
+          <t>סוג הפקודה מגדיר פרמטרים, טווח מספרים ופרופיל סטטוס</t>
         </is>
       </c>
       <c r="J42" s="107">
-        <f>HYPERLINK("#'"&amp;"8. ניהול סטטוסים (Status Mgmt)"&amp;"'!A9","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"12. היסטוריה וארכיון"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60798,12 +60939,12 @@
       </c>
       <c r="B43" s="102" t="inlineStr">
         <is>
-          <t>T003O</t>
+          <t>JEST</t>
         </is>
       </c>
       <c r="C43" s="102" t="inlineStr">
         <is>
-          <t>STSMA</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="D43" s="96" t="inlineStr">
@@ -60813,12 +60954,12 @@
       </c>
       <c r="E43" s="44" t="inlineStr">
         <is>
-          <t>TJ30</t>
+          <t>JSTO</t>
         </is>
       </c>
       <c r="F43" s="44" t="inlineStr">
         <is>
-          <t>STSMA</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="G43" s="96" t="inlineStr">
@@ -60828,16 +60969,16 @@
       </c>
       <c r="H43" s="104" t="inlineStr">
         <is>
-          <t>T003O.STSMA = TJ30.STSMA</t>
+          <t>JEST.OBJNR = JSTO.OBJNR</t>
         </is>
       </c>
       <c r="I43" s="46" t="inlineStr">
         <is>
-          <t>פרופיל הסטטוס המשויך לסוג הפקודה</t>
+          <t>סטטוסים פעילים תחת אובייקט הסטטוס</t>
         </is>
       </c>
       <c r="J43" s="105">
-        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A45","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"8. ניהול סטטוסים (Status Mgmt)"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60847,12 +60988,12 @@
       </c>
       <c r="B44" s="103" t="inlineStr">
         <is>
-          <t>RESB</t>
+          <t>JSTO</t>
         </is>
       </c>
       <c r="C44" s="103" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>STSMA</t>
         </is>
       </c>
       <c r="D44" s="100" t="inlineStr">
@@ -60862,12 +61003,12 @@
       </c>
       <c r="E44" s="52" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>TJ30</t>
         </is>
       </c>
       <c r="F44" s="52" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>STSMA</t>
         </is>
       </c>
       <c r="G44" s="100" t="inlineStr">
@@ -60877,16 +61018,16 @@
       </c>
       <c r="H44" s="106" t="inlineStr">
         <is>
-          <t>RESB.AUFNR = AUFK.AUFNR</t>
+          <t>JSTO.STSMA = TJ30.STSMA</t>
         </is>
       </c>
       <c r="I44" s="54" t="inlineStr">
         <is>
-          <t>הזמנות רכיבים של הפק"ע</t>
+          <t>פרופיל הסטטוס מגדיר את סטטוסי המשתמש</t>
         </is>
       </c>
       <c r="J44" s="107">
-        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A3","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"8. ניהול סטטוסים (Status Mgmt)"&amp;"'!A9","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60896,12 +61037,12 @@
       </c>
       <c r="B45" s="102" t="inlineStr">
         <is>
-          <t>MSEG</t>
+          <t>T003O</t>
         </is>
       </c>
       <c r="C45" s="102" t="inlineStr">
         <is>
-          <t>MBLNR</t>
+          <t>STSMA</t>
         </is>
       </c>
       <c r="D45" s="96" t="inlineStr">
@@ -60911,12 +61052,12 @@
       </c>
       <c r="E45" s="44" t="inlineStr">
         <is>
-          <t>MKPF</t>
+          <t>TJ30</t>
         </is>
       </c>
       <c r="F45" s="44" t="inlineStr">
         <is>
-          <t>MBLNR</t>
+          <t>STSMA</t>
         </is>
       </c>
       <c r="G45" s="96" t="inlineStr">
@@ -60926,16 +61067,16 @@
       </c>
       <c r="H45" s="104" t="inlineStr">
         <is>
-          <t>MSEG.MBLNR = MKPF.MBLNR</t>
+          <t>T003O.STSMA = TJ30.STSMA</t>
         </is>
       </c>
       <c r="I45" s="46" t="inlineStr">
         <is>
-          <t>פריטי מסמך החומר תחת הכותרת</t>
+          <t>פרופיל הסטטוס המשויך לסוג הפקודה</t>
         </is>
       </c>
       <c r="J45" s="105">
-        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A25","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"7. פקודות עבודה (פק"ע)"&amp;"'!A45","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60945,7 +61086,7 @@
       </c>
       <c r="B46" s="103" t="inlineStr">
         <is>
-          <t>MSEG</t>
+          <t>RESB</t>
         </is>
       </c>
       <c r="C46" s="103" t="inlineStr">
@@ -60975,16 +61116,16 @@
       </c>
       <c r="H46" s="106" t="inlineStr">
         <is>
-          <t>MSEG.AUFNR = AUFK.AUFNR</t>
+          <t>RESB.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="I46" s="54" t="inlineStr">
         <is>
-          <t>תנועת המלאי מחויבת לפק"ע</t>
+          <t>הזמנות רכיבים של הפק"ע</t>
         </is>
       </c>
       <c r="J46" s="107">
-        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A25","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -60994,12 +61135,12 @@
       </c>
       <c r="B47" s="102" t="inlineStr">
         <is>
-          <t>EBKN</t>
+          <t>MSEG</t>
         </is>
       </c>
       <c r="C47" s="102" t="inlineStr">
         <is>
-          <t>BANFN</t>
+          <t>MBLNR</t>
         </is>
       </c>
       <c r="D47" s="96" t="inlineStr">
@@ -61009,12 +61150,12 @@
       </c>
       <c r="E47" s="44" t="inlineStr">
         <is>
-          <t>EBAN</t>
+          <t>MKPF</t>
         </is>
       </c>
       <c r="F47" s="44" t="inlineStr">
         <is>
-          <t>BANFN</t>
+          <t>MBLNR</t>
         </is>
       </c>
       <c r="G47" s="96" t="inlineStr">
@@ -61024,16 +61165,16 @@
       </c>
       <c r="H47" s="104" t="inlineStr">
         <is>
-          <t>EBKN.BANFN = EBAN.BANFN</t>
+          <t>MSEG.MBLNR = MKPF.MBLNR</t>
         </is>
       </c>
       <c r="I47" s="46" t="inlineStr">
         <is>
-          <t>חיוב דרישת הרכש</t>
+          <t>פריטי מסמך החומר תחת הכותרת</t>
         </is>
       </c>
       <c r="J47" s="105">
-        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A18","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61043,7 +61184,7 @@
       </c>
       <c r="B48" s="103" t="inlineStr">
         <is>
-          <t>EBKN</t>
+          <t>MSEG</t>
         </is>
       </c>
       <c r="C48" s="103" t="inlineStr">
@@ -61073,16 +61214,16 @@
       </c>
       <c r="H48" s="106" t="inlineStr">
         <is>
-          <t>EBKN.AUFNR = AUFK.AUFNR</t>
+          <t>MSEG.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="I48" s="54" t="inlineStr">
         <is>
-          <t>דרישת הרכש מחויבת לפק"ע</t>
+          <t>תנועת המלאי מחויבת לפק"ע</t>
         </is>
       </c>
       <c r="J48" s="107">
-        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A18","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61092,12 +61233,12 @@
       </c>
       <c r="B49" s="102" t="inlineStr">
         <is>
-          <t>COSP</t>
+          <t>EBKN</t>
         </is>
       </c>
       <c r="C49" s="102" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>BANFN</t>
         </is>
       </c>
       <c r="D49" s="96" t="inlineStr">
@@ -61107,12 +61248,12 @@
       </c>
       <c r="E49" s="44" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>EBAN</t>
         </is>
       </c>
       <c r="F49" s="44" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>BANFN</t>
         </is>
       </c>
       <c r="G49" s="96" t="inlineStr">
@@ -61122,16 +61263,16 @@
       </c>
       <c r="H49" s="104" t="inlineStr">
         <is>
-          <t>COSP.OBJNR = AUFK.OBJNR</t>
+          <t>EBKN.BANFN = EBAN.BANFN</t>
         </is>
       </c>
       <c r="I49" s="46" t="inlineStr">
         <is>
-          <t>סך עלויות חיצוניות לפי אובייקט הפק"ע</t>
+          <t>חיוב דרישת הרכש</t>
         </is>
       </c>
       <c r="J49" s="105">
-        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A3","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A18","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61141,12 +61282,12 @@
       </c>
       <c r="B50" s="103" t="inlineStr">
         <is>
-          <t>COSS</t>
+          <t>EBKN</t>
         </is>
       </c>
       <c r="C50" s="103" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>AUFNR</t>
         </is>
       </c>
       <c r="D50" s="100" t="inlineStr">
@@ -61161,7 +61302,7 @@
       </c>
       <c r="F50" s="52" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>AUFNR</t>
         </is>
       </c>
       <c r="G50" s="100" t="inlineStr">
@@ -61171,16 +61312,16 @@
       </c>
       <c r="H50" s="106" t="inlineStr">
         <is>
-          <t>COSS.OBJNR = AUFK.OBJNR</t>
+          <t>EBKN.AUFNR = AUFK.AUFNR</t>
         </is>
       </c>
       <c r="I50" s="54" t="inlineStr">
         <is>
-          <t>סך עלויות פנימיות לפי אובייקט הפק"ע</t>
+          <t>דרישת הרכש מחויבת לפק"ע</t>
         </is>
       </c>
       <c r="J50" s="107">
-        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A10","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A18","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61190,12 +61331,12 @@
       </c>
       <c r="B51" s="102" t="inlineStr">
         <is>
-          <t>COBRA</t>
+          <t>EBAN</t>
         </is>
       </c>
       <c r="C51" s="102" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>FLIEF</t>
         </is>
       </c>
       <c r="D51" s="96" t="inlineStr">
@@ -61205,31 +61346,31 @@
       </c>
       <c r="E51" s="44" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>BUT000</t>
         </is>
       </c>
       <c r="F51" s="44" t="inlineStr">
         <is>
-          <t>OBJNR</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="G51" s="96" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>N:1</t>
         </is>
       </c>
       <c r="H51" s="104" t="inlineStr">
         <is>
-          <t>COBRA.OBJNR = AUFK.OBJNR</t>
+          <t>EBAN.FLIEF = BUT000.PARTNER</t>
         </is>
       </c>
       <c r="I51" s="46" t="inlineStr">
         <is>
-          <t>כותרת חוק ההתחשבנות של הפק"ע</t>
+          <t>ספק קבוע בדרישת הרכש - ב-S/4 דרך Business Partner (CVI)</t>
         </is>
       </c>
       <c r="J51" s="105">
-        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A17","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"9. אינטגרציית מלאי ורכש (PM-MM)"&amp;"'!A11","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61239,7 +61380,7 @@
       </c>
       <c r="B52" s="103" t="inlineStr">
         <is>
-          <t>COBRB</t>
+          <t>COSP</t>
         </is>
       </c>
       <c r="C52" s="103" t="inlineStr">
@@ -61254,7 +61395,7 @@
       </c>
       <c r="E52" s="52" t="inlineStr">
         <is>
-          <t>COBRA</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="F52" s="52" t="inlineStr">
@@ -61269,16 +61410,16 @@
       </c>
       <c r="H52" s="106" t="inlineStr">
         <is>
-          <t>COBRB.OBJNR = COBRA.OBJNR</t>
+          <t>COSP.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="I52" s="54" t="inlineStr">
         <is>
-          <t>פריטי חוק ההתחשבנות (חוקי חלוקה)</t>
+          <t>סך עלויות חיצוניות לפי אובייקט הפק"ע</t>
         </is>
       </c>
       <c r="J52" s="107">
-        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A23","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A3","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61288,12 +61429,12 @@
       </c>
       <c r="B53" s="102" t="inlineStr">
         <is>
-          <t>MPOS</t>
+          <t>COSS</t>
         </is>
       </c>
       <c r="C53" s="102" t="inlineStr">
         <is>
-          <t>WARPL</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="D53" s="96" t="inlineStr">
@@ -61303,12 +61444,12 @@
       </c>
       <c r="E53" s="44" t="inlineStr">
         <is>
-          <t>MPLA</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="F53" s="44" t="inlineStr">
         <is>
-          <t>WARPL</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="G53" s="96" t="inlineStr">
@@ -61318,16 +61459,16 @@
       </c>
       <c r="H53" s="104" t="inlineStr">
         <is>
-          <t>MPOS.WARPL = MPLA.WARPL</t>
+          <t>COSS.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="I53" s="46" t="inlineStr">
         <is>
-          <t>פריטי תכנית האחזקה</t>
+          <t>סך עלויות פנימיות לפי אובייקט הפק"ע</t>
         </is>
       </c>
       <c r="J53" s="105">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61337,12 +61478,12 @@
       </c>
       <c r="B54" s="103" t="inlineStr">
         <is>
-          <t>MPOS</t>
+          <t>COBRA</t>
         </is>
       </c>
       <c r="C54" s="103" t="inlineStr">
         <is>
-          <t>EQUNR</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="D54" s="100" t="inlineStr">
@@ -61352,31 +61493,31 @@
       </c>
       <c r="E54" s="52" t="inlineStr">
         <is>
-          <t>EQUI</t>
+          <t>AUFK</t>
         </is>
       </c>
       <c r="F54" s="52" t="inlineStr">
         <is>
-          <t>EQUNR</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="G54" s="100" t="inlineStr">
         <is>
-          <t>N:1</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="H54" s="106" t="inlineStr">
         <is>
-          <t>MPOS.EQUNR = EQUI.EQUNR</t>
+          <t>COBRA.OBJNR = AUFK.OBJNR</t>
         </is>
       </c>
       <c r="I54" s="54" t="inlineStr">
         <is>
-          <t>פריט התכנית מתייחס לציוד</t>
+          <t>כותרת חוק ההתחשבנות של הפק"ע</t>
         </is>
       </c>
       <c r="J54" s="107">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A17","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61386,12 +61527,12 @@
       </c>
       <c r="B55" s="102" t="inlineStr">
         <is>
-          <t>MPOS</t>
+          <t>COBRB</t>
         </is>
       </c>
       <c r="C55" s="102" t="inlineStr">
         <is>
-          <t>PLNNR</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="D55" s="96" t="inlineStr">
@@ -61401,12 +61542,12 @@
       </c>
       <c r="E55" s="44" t="inlineStr">
         <is>
-          <t>PLKO</t>
+          <t>COBRA</t>
         </is>
       </c>
       <c r="F55" s="44" t="inlineStr">
         <is>
-          <t>PLNNR</t>
+          <t>OBJNR</t>
         </is>
       </c>
       <c r="G55" s="96" t="inlineStr">
@@ -61416,16 +61557,16 @@
       </c>
       <c r="H55" s="104" t="inlineStr">
         <is>
-          <t>MPOS.PLNNR = PLKO.PLNNR</t>
+          <t>COBRB.OBJNR = COBRA.OBJNR</t>
         </is>
       </c>
       <c r="I55" s="46" t="inlineStr">
         <is>
-          <t>רשימת הפעולות המשויכת לפריט</t>
+          <t>פריטי חוק ההתחשבנות (חוקי חלוקה)</t>
         </is>
       </c>
       <c r="J55" s="105">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"10. עלויות והתחשבנות (PM-CO)"&amp;"'!A23","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61435,7 +61576,7 @@
       </c>
       <c r="B56" s="103" t="inlineStr">
         <is>
-          <t>MHIO</t>
+          <t>MPOS</t>
         </is>
       </c>
       <c r="C56" s="103" t="inlineStr">
@@ -61465,16 +61606,16 @@
       </c>
       <c r="H56" s="106" t="inlineStr">
         <is>
-          <t>MHIO.WARPL = MPLA.WARPL</t>
+          <t>MPOS.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="I56" s="54" t="inlineStr">
         <is>
-          <t>אובייקטי קריאת התכנית</t>
+          <t>פריטי תכנית האחזקה</t>
         </is>
       </c>
       <c r="J56" s="107">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A33","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61484,12 +61625,12 @@
       </c>
       <c r="B57" s="102" t="inlineStr">
         <is>
-          <t>MHIO</t>
+          <t>MPOS</t>
         </is>
       </c>
       <c r="C57" s="102" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>EQUNR</t>
         </is>
       </c>
       <c r="D57" s="96" t="inlineStr">
@@ -61499,12 +61640,12 @@
       </c>
       <c r="E57" s="44" t="inlineStr">
         <is>
-          <t>AUFK</t>
+          <t>EQUI</t>
         </is>
       </c>
       <c r="F57" s="44" t="inlineStr">
         <is>
-          <t>AUFNR</t>
+          <t>EQUNR</t>
         </is>
       </c>
       <c r="G57" s="96" t="inlineStr">
@@ -61514,16 +61655,16 @@
       </c>
       <c r="H57" s="104" t="inlineStr">
         <is>
-          <t>MHIO.AUFNR = AUFK.AUFNR</t>
+          <t>MPOS.EQUNR = EQUI.EQUNR</t>
         </is>
       </c>
       <c r="I57" s="46" t="inlineStr">
         <is>
-          <t>הפק"ע שנוצרה מהקריאה</t>
+          <t>פריט התכנית מתייחס לציוד</t>
         </is>
       </c>
       <c r="J57" s="105">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A33","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61533,12 +61674,12 @@
       </c>
       <c r="B58" s="103" t="inlineStr">
         <is>
-          <t>MHIS</t>
+          <t>MPOS</t>
         </is>
       </c>
       <c r="C58" s="103" t="inlineStr">
         <is>
-          <t>WARPL</t>
+          <t>PLNNR</t>
         </is>
       </c>
       <c r="D58" s="100" t="inlineStr">
@@ -61548,12 +61689,12 @@
       </c>
       <c r="E58" s="52" t="inlineStr">
         <is>
-          <t>MPLA</t>
+          <t>PLKO</t>
         </is>
       </c>
       <c r="F58" s="52" t="inlineStr">
         <is>
-          <t>WARPL</t>
+          <t>PLNNR</t>
         </is>
       </c>
       <c r="G58" s="100" t="inlineStr">
@@ -61563,16 +61704,16 @@
       </c>
       <c r="H58" s="106" t="inlineStr">
         <is>
-          <t>MHIS.WARPL = MPLA.WARPL</t>
+          <t>MPOS.PLNNR = PLKO.PLNNR</t>
         </is>
       </c>
       <c r="I58" s="54" t="inlineStr">
         <is>
-          <t>היסטוריית התזמון של התכנית</t>
+          <t>רשימת הפעולות המשויכת לפריט</t>
         </is>
       </c>
       <c r="J58" s="107">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A40","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A25","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61582,12 +61723,12 @@
       </c>
       <c r="B59" s="102" t="inlineStr">
         <is>
-          <t>PLPO</t>
+          <t>MHIO</t>
         </is>
       </c>
       <c r="C59" s="102" t="inlineStr">
         <is>
-          <t>PLNNR</t>
+          <t>WARPL</t>
         </is>
       </c>
       <c r="D59" s="96" t="inlineStr">
@@ -61597,12 +61738,12 @@
       </c>
       <c r="E59" s="44" t="inlineStr">
         <is>
-          <t>PLKO</t>
+          <t>MPLA</t>
         </is>
       </c>
       <c r="F59" s="44" t="inlineStr">
         <is>
-          <t>PLNNR</t>
+          <t>WARPL</t>
         </is>
       </c>
       <c r="G59" s="96" t="inlineStr">
@@ -61612,16 +61753,16 @@
       </c>
       <c r="H59" s="104" t="inlineStr">
         <is>
-          <t>PLPO.PLNNR = PLKO.PLNNR</t>
+          <t>MHIO.WARPL = MPLA.WARPL</t>
         </is>
       </c>
       <c r="I59" s="46" t="inlineStr">
         <is>
-          <t>פעולות רשימת הפעולות תחת הכותרת</t>
+          <t>אובייקטי קריאת התכנית</t>
         </is>
       </c>
       <c r="J59" s="105">
-        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A10","➜ פתח")</f>
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A33","➜ פתח")</f>
         <v/>
       </c>
     </row>
@@ -61631,45 +61772,192 @@
       </c>
       <c r="B60" s="103" t="inlineStr">
         <is>
+          <t>MHIO</t>
+        </is>
+      </c>
+      <c r="C60" s="103" t="inlineStr">
+        <is>
+          <t>AUFNR</t>
+        </is>
+      </c>
+      <c r="D60" s="100" t="inlineStr">
+        <is>
+          <t>➜</t>
+        </is>
+      </c>
+      <c r="E60" s="52" t="inlineStr">
+        <is>
+          <t>AUFK</t>
+        </is>
+      </c>
+      <c r="F60" s="52" t="inlineStr">
+        <is>
+          <t>AUFNR</t>
+        </is>
+      </c>
+      <c r="G60" s="100" t="inlineStr">
+        <is>
+          <t>N:1</t>
+        </is>
+      </c>
+      <c r="H60" s="106" t="inlineStr">
+        <is>
+          <t>MHIO.AUFNR = AUFK.AUFNR</t>
+        </is>
+      </c>
+      <c r="I60" s="54" t="inlineStr">
+        <is>
+          <t>הפק"ע שנוצרה מהקריאה</t>
+        </is>
+      </c>
+      <c r="J60" s="107">
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A33","➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="96" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="102" t="inlineStr">
+        <is>
+          <t>MHIS</t>
+        </is>
+      </c>
+      <c r="C61" s="102" t="inlineStr">
+        <is>
+          <t>WARPL</t>
+        </is>
+      </c>
+      <c r="D61" s="96" t="inlineStr">
+        <is>
+          <t>➜</t>
+        </is>
+      </c>
+      <c r="E61" s="44" t="inlineStr">
+        <is>
+          <t>MPLA</t>
+        </is>
+      </c>
+      <c r="F61" s="44" t="inlineStr">
+        <is>
+          <t>WARPL</t>
+        </is>
+      </c>
+      <c r="G61" s="96" t="inlineStr">
+        <is>
+          <t>N:1</t>
+        </is>
+      </c>
+      <c r="H61" s="104" t="inlineStr">
+        <is>
+          <t>MHIS.WARPL = MPLA.WARPL</t>
+        </is>
+      </c>
+      <c r="I61" s="46" t="inlineStr">
+        <is>
+          <t>היסטוריית התזמון של התכנית</t>
+        </is>
+      </c>
+      <c r="J61" s="105">
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A40","➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="24" customHeight="1">
+      <c r="A62" s="100" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="103" t="inlineStr">
+        <is>
           <t>PLPO</t>
         </is>
       </c>
-      <c r="C60" s="103" t="inlineStr">
+      <c r="C62" s="103" t="inlineStr">
+        <is>
+          <t>PLNNR</t>
+        </is>
+      </c>
+      <c r="D62" s="100" t="inlineStr">
+        <is>
+          <t>➜</t>
+        </is>
+      </c>
+      <c r="E62" s="52" t="inlineStr">
+        <is>
+          <t>PLKO</t>
+        </is>
+      </c>
+      <c r="F62" s="52" t="inlineStr">
+        <is>
+          <t>PLNNR</t>
+        </is>
+      </c>
+      <c r="G62" s="100" t="inlineStr">
+        <is>
+          <t>N:1</t>
+        </is>
+      </c>
+      <c r="H62" s="106" t="inlineStr">
+        <is>
+          <t>PLPO.PLNNR = PLKO.PLNNR</t>
+        </is>
+      </c>
+      <c r="I62" s="54" t="inlineStr">
+        <is>
+          <t>פעולות רשימת הפעולות תחת הכותרת</t>
+        </is>
+      </c>
+      <c r="J62" s="107">
+        <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A10","➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="24" customHeight="1">
+      <c r="A63" s="96" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="102" t="inlineStr">
+        <is>
+          <t>PLPO</t>
+        </is>
+      </c>
+      <c r="C63" s="102" t="inlineStr">
         <is>
           <t>ARBID</t>
         </is>
       </c>
-      <c r="D60" s="100" t="inlineStr">
+      <c r="D63" s="96" t="inlineStr">
         <is>
           <t>➜</t>
         </is>
       </c>
-      <c r="E60" s="52" t="inlineStr">
+      <c r="E63" s="44" t="inlineStr">
         <is>
           <t>CRHD</t>
         </is>
       </c>
-      <c r="F60" s="52" t="inlineStr">
+      <c r="F63" s="44" t="inlineStr">
         <is>
           <t>OBJID</t>
         </is>
       </c>
-      <c r="G60" s="100" t="inlineStr">
+      <c r="G63" s="96" t="inlineStr">
         <is>
           <t>N:1</t>
         </is>
       </c>
-      <c r="H60" s="106" t="inlineStr">
+      <c r="H63" s="104" t="inlineStr">
         <is>
           <t>PLPO.ARBID = CRHD.OBJID</t>
         </is>
       </c>
-      <c r="I60" s="54" t="inlineStr">
+      <c r="I63" s="46" t="inlineStr">
         <is>
           <t>מרכז העבודה של הפעולה ברשימה</t>
         </is>
       </c>
-      <c r="J60" s="107">
+      <c r="J63" s="105">
         <f>HYPERLINK("#'"&amp;"11. אחזקה מונעת ותוכניות"&amp;"'!A10","➜ פתח")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add encyclopedic Config Guide sheet: Hebrew configuration guides, HE/EN terminology, official SAP Help/Note/SIC/Fiori links for config objects (T003O/T356/TQ80/TJ30/TJ30T/BUT000)
</commit_message>
<xml_diff>
--- a/SAP_PM_ECC6_to_S4_Migration.xlsx
+++ b/SAP_PM_ECC6_to_S4_Migration.xlsx
@@ -24,9 +24,10 @@
     <sheet name="Cockpit מעקב מיגרציה" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Custom Code Check" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="ER - Join Map" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Config Guide" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'מסך ניווט מרכזי'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'מסך ניווט מרכזי'!$A$1:$O$64</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1. מבנה ארגוני ותשתית'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'1. מבנה ארגוני ותשתית'!$A$1:$P$53</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'2. ציוד ונתוני מאסטר'!$1:$2</definedName>
@@ -59,6 +60,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="15">'Custom Code Check'!$A$1:$I$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="16">'ER - Join Map'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="16">'ER - Join Map'!$A$1:$J$63</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="17">'Config Guide'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="17">'Config Guide'!$A$1:$G$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +70,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="64">
+  <fonts count="65">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -268,6 +271,13 @@
       <b val="1"/>
       <color rgb="000B5394"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -611,51 +621,51 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="55" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="56" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="40" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="40" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="41" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -682,33 +692,33 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="44" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="61" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="12" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="62" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="62" fillId="12" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="63" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="64" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="55" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -751,7 +761,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -770,7 +780,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -917,6 +927,24 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1358,7 +1386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V909"/>
+  <dimension ref="A1:V915"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2586,17 +2614,17 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="29" t="inlineStr">
-        <is>
-          <t>מקרא מותג CBC:  אדום=תנועתי/עוגני-על | צפחה=נתוני אב וכותרות | כסף=אינטגרציה ועמודות S/4HANA</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>📖 Config Guide</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
+      <c r="E22" s="1" t="n"/>
+      <c r="F22" s="1" t="n"/>
+      <c r="G22" s="1" t="n"/>
+      <c r="H22" s="1" t="n"/>
       <c r="I22" s="1" t="n"/>
       <c r="J22" s="1" t="n"/>
       <c r="K22" s="1" t="n"/>
@@ -2641,7 +2669,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="1" t="n"/>
+      <c r="B23" s="26" t="n"/>
       <c r="C23" s="1" t="n"/>
       <c r="D23" s="1" t="n"/>
       <c r="E23" s="1" t="n"/>
@@ -2692,15 +2720,11 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="24" t="inlineStr">
-        <is>
-          <t>🔍 חיפוש גלובלי  (טבלה / טרנזקציה / שדה / פונקציה - עברית או אנגלית)</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
+      <c r="B24" s="1" t="n"/>
+      <c r="C24" s="1" t="n"/>
+      <c r="D24" s="1" t="n"/>
+      <c r="E24" s="1" t="n"/>
+      <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
       <c r="H24" s="1" t="n"/>
       <c r="I24" s="1" t="n"/>
@@ -2745,19 +2769,19 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
+    <row r="25">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>הקלד כאן:</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr"/>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>מקרא מותג CBC:  אדום=תנועתי/עוגני-על | צפחה=נתוני אב וכותרות | כסף=אינטגרציה ועמודות S/4HANA</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="1" t="n"/>
-      <c r="H25" s="1" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
       <c r="I25" s="1" t="n"/>
       <c r="J25" s="1" t="n"/>
       <c r="K25" s="1" t="n"/>
@@ -2853,36 +2877,16 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="32" t="inlineStr">
-        <is>
-          <t>קישור</t>
-        </is>
-      </c>
-      <c r="C27" s="32" t="inlineStr">
-        <is>
-          <t>קוד / שם טכני</t>
-        </is>
-      </c>
-      <c r="D27" s="32" t="inlineStr">
-        <is>
-          <t>פירוש בעברית</t>
-        </is>
-      </c>
-      <c r="E27" s="32" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F27" s="32" t="inlineStr">
-        <is>
-          <t>גיליון</t>
-        </is>
-      </c>
-      <c r="G27" s="32" t="inlineStr">
-        <is>
-          <t>תא</t>
-        </is>
-      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>🔍 חיפוש גלובלי  (טבלה / טרנזקציה / שדה / פונקציה - עברית או אנגלית)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="1" t="n"/>
       <c r="H27" s="1" t="n"/>
       <c r="I27" s="1" t="n"/>
       <c r="J27" s="1" t="n"/>
@@ -2926,16 +2930,17 @@
         <v/>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="26" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="33">
-        <f>IF(C25="","הקלד מונח בתא הצהוב למעלה - והתוצאות יופיעו כאן מיד (כולל קישור לחיץ)...",IFERROR(_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6},$V$2:$V$909,$Q$2:$Q$909,$R$2:$R$909,$S$2:$S$909,$T$2:$T$909,$U$2:$U$909),(ISNUMBER(SEARCH(C25,$Q$2:$Q$909)))+(ISNUMBER(SEARCH(C25,$R$2:$R$909)))+(ISNUMBER(SEARCH(C25,$S$2:$S$909)))+(ISNUMBER(SEARCH(C25,$P$2:$P$909)))&gt;0),"לא נמצאו תוצאות - נסה מונח אחר"))</f>
-        <v/>
-      </c>
-      <c r="C28" s="1" t="n"/>
-      <c r="D28" s="1" t="n"/>
-      <c r="E28" s="1" t="n"/>
-      <c r="F28" s="1" t="n"/>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>הקלד כאן:</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
       <c r="G28" s="1" t="n"/>
       <c r="H28" s="1" t="n"/>
       <c r="I28" s="1" t="n"/>
@@ -3033,12 +3038,36 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="1" t="n"/>
-      <c r="C30" s="1" t="n"/>
-      <c r="D30" s="1" t="n"/>
-      <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="n"/>
-      <c r="G30" s="1" t="n"/>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>קישור</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="inlineStr">
+        <is>
+          <t>קוד / שם טכני</t>
+        </is>
+      </c>
+      <c r="D30" s="32" t="inlineStr">
+        <is>
+          <t>פירוש בעברית</t>
+        </is>
+      </c>
+      <c r="E30" s="32" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F30" s="32" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="G30" s="32" t="inlineStr">
+        <is>
+          <t>תא</t>
+        </is>
+      </c>
       <c r="H30" s="1" t="n"/>
       <c r="I30" s="1" t="n"/>
       <c r="J30" s="1" t="n"/>
@@ -3084,7 +3113,10 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
+      <c r="B31" s="33">
+        <f>IF(C28="","הקלד מונח בתא הצהוב למעלה - והתוצאות יופיעו כאן מיד (כולל קישור לחיץ)...",IFERROR(_xlfn._xlws.FILTER(CHOOSE({1,2,3,4,5,6},$V$2:$V$915,$Q$2:$Q$915,$R$2:$R$915,$S$2:$S$915,$T$2:$T$915,$U$2:$U$915),(ISNUMBER(SEARCH(C28,$Q$2:$Q$915)))+(ISNUMBER(SEARCH(C28,$R$2:$R$915)))+(ISNUMBER(SEARCH(C28,$S$2:$S$915)))+(ISNUMBER(SEARCH(C28,$P$2:$P$915)))&gt;0),"לא נמצאו תוצאות - נסה מונח אחר"))</f>
+        <v/>
+      </c>
       <c r="C31" s="1" t="n"/>
       <c r="D31" s="1" t="n"/>
       <c r="E31" s="1" t="n"/>
@@ -4359,17 +4391,13 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n"/>
-      <c r="B56" s="34" t="inlineStr">
-        <is>
-          <t>איך עובדים:  1) לחץ כרטיס למעבר לגיליון (כולל Cockpit מעקב מיגרציה ו-Custom Code Check).  2) הקלד מונח בתא הצהוב - התוצאות הדינמיות (FILTER) יופיעו מיד עם קישור לחיץ לשורה.  3) בכל גיליון יש כפתור 'חזרה למסך הראשי' בפינה הימנית-עליונה (קישור Hyperlink).  ב-Cockpit וב-Custom Code Check יש עמודות סטטוס עם רשימה נפתחת וצביעה אוטומטית.  קובץ זה הוא .xlsx נקי (ללא מאקרו) - בטוח למייל ארגוני. להוספת כפתור חיפוש-מאקרו: הדבק את modPM.bas דרך Alt+F11 ושמור כ-.xlsm (הוראות מצורפות).</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
-      <c r="H56" s="4" t="n"/>
+      <c r="B56" s="1" t="n"/>
+      <c r="C56" s="1" t="n"/>
+      <c r="D56" s="1" t="n"/>
+      <c r="E56" s="1" t="n"/>
+      <c r="F56" s="1" t="n"/>
+      <c r="G56" s="1" t="n"/>
+      <c r="H56" s="1" t="n"/>
       <c r="I56" s="1" t="n"/>
       <c r="J56" s="1" t="n"/>
       <c r="K56" s="1" t="n"/>
@@ -4414,13 +4442,13 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="4" t="n"/>
+      <c r="B57" s="1" t="n"/>
+      <c r="C57" s="1" t="n"/>
+      <c r="D57" s="1" t="n"/>
+      <c r="E57" s="1" t="n"/>
+      <c r="F57" s="1" t="n"/>
+      <c r="G57" s="1" t="n"/>
+      <c r="H57" s="1" t="n"/>
       <c r="I57" s="1" t="n"/>
       <c r="J57" s="1" t="n"/>
       <c r="K57" s="1" t="n"/>
@@ -4465,7 +4493,11 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n"/>
-      <c r="B58" s="4" t="n"/>
+      <c r="B58" s="34" t="inlineStr">
+        <is>
+          <t>איך עובדים:  1) לחץ כרטיס למעבר לגיליון (כולל Cockpit מעקב מיגרציה ו-Custom Code Check).  2) הקלד מונח בתא הצהוב - התוצאות הדינמיות (FILTER) יופיעו מיד עם קישור לחיץ לשורה.  3) בכל גיליון יש כפתור 'חזרה למסך הראשי' בפינה הימנית-עליונה (קישור Hyperlink).  ב-Cockpit וב-Custom Code Check יש עמודות סטטוס עם רשימה נפתחת וצביעה אוטומטית.  קובץ זה הוא .xlsx נקי (ללא מאקרו) - בטוח למייל ארגוני. להוספת כפתור חיפוש-מאקרו: הדבק את modPM.bas דרך Alt+F11 ושמור כ-.xlsm (הוראות מצורפות).</t>
+        </is>
+      </c>
       <c r="C58" s="4" t="n"/>
       <c r="D58" s="4" t="n"/>
       <c r="E58" s="4" t="n"/>
@@ -4618,13 +4650,13 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n"/>
-      <c r="B61" s="1" t="n"/>
-      <c r="C61" s="1" t="n"/>
-      <c r="D61" s="1" t="n"/>
-      <c r="E61" s="1" t="n"/>
-      <c r="F61" s="1" t="n"/>
-      <c r="G61" s="1" t="n"/>
-      <c r="H61" s="1" t="n"/>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="4" t="n"/>
+      <c r="D61" s="4" t="n"/>
+      <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="n"/>
+      <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
       <c r="I61" s="1" t="n"/>
       <c r="J61" s="1" t="n"/>
       <c r="K61" s="1" t="n"/>
@@ -4669,13 +4701,13 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n"/>
-      <c r="B62" s="1" t="n"/>
-      <c r="C62" s="1" t="n"/>
-      <c r="D62" s="1" t="n"/>
-      <c r="E62" s="1" t="n"/>
-      <c r="F62" s="1" t="n"/>
-      <c r="G62" s="1" t="n"/>
-      <c r="H62" s="1" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
       <c r="I62" s="1" t="n"/>
       <c r="J62" s="1" t="n"/>
       <c r="K62" s="1" t="n"/>
@@ -4719,21 +4751,21 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="n"/>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="n"/>
-      <c r="I63" s="4" t="n"/>
-      <c r="J63" s="4" t="n"/>
-      <c r="K63" s="4" t="n"/>
-      <c r="L63" s="4" t="n"/>
-      <c r="M63" s="4" t="n"/>
-      <c r="N63" s="4" t="n"/>
-      <c r="O63" s="4" t="n"/>
+      <c r="A63" s="1" t="n"/>
+      <c r="B63" s="1" t="n"/>
+      <c r="C63" s="1" t="n"/>
+      <c r="D63" s="1" t="n"/>
+      <c r="E63" s="1" t="n"/>
+      <c r="F63" s="1" t="n"/>
+      <c r="G63" s="1" t="n"/>
+      <c r="H63" s="1" t="n"/>
+      <c r="I63" s="1" t="n"/>
+      <c r="J63" s="1" t="n"/>
+      <c r="K63" s="1" t="n"/>
+      <c r="L63" s="1" t="n"/>
+      <c r="M63" s="1" t="n"/>
+      <c r="N63" s="1" t="n"/>
+      <c r="O63" s="1" t="n"/>
       <c r="P63" s="7" t="inlineStr">
         <is>
           <t>תוכנית</t>
@@ -4770,21 +4802,21 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="n"/>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="n"/>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n"/>
-      <c r="M64" s="4" t="n"/>
-      <c r="N64" s="4" t="n"/>
-      <c r="O64" s="4" t="n"/>
+      <c r="A64" s="1" t="n"/>
+      <c r="B64" s="1" t="n"/>
+      <c r="C64" s="1" t="n"/>
+      <c r="D64" s="1" t="n"/>
+      <c r="E64" s="1" t="n"/>
+      <c r="F64" s="1" t="n"/>
+      <c r="G64" s="1" t="n"/>
+      <c r="H64" s="1" t="n"/>
+      <c r="I64" s="1" t="n"/>
+      <c r="J64" s="1" t="n"/>
+      <c r="K64" s="1" t="n"/>
+      <c r="L64" s="1" t="n"/>
+      <c r="M64" s="1" t="n"/>
+      <c r="N64" s="1" t="n"/>
+      <c r="O64" s="1" t="n"/>
       <c r="P64" s="7" t="inlineStr">
         <is>
           <t>Fiori</t>
@@ -4821,21 +4853,21 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="n"/>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="n"/>
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="4" t="n"/>
-      <c r="H65" s="4" t="n"/>
-      <c r="I65" s="4" t="n"/>
-      <c r="J65" s="4" t="n"/>
-      <c r="K65" s="4" t="n"/>
-      <c r="L65" s="4" t="n"/>
-      <c r="M65" s="4" t="n"/>
-      <c r="N65" s="4" t="n"/>
-      <c r="O65" s="4" t="n"/>
+      <c r="A65" s="1" t="n"/>
+      <c r="B65" s="1" t="n"/>
+      <c r="C65" s="1" t="n"/>
+      <c r="D65" s="1" t="n"/>
+      <c r="E65" s="1" t="n"/>
+      <c r="F65" s="1" t="n"/>
+      <c r="G65" s="1" t="n"/>
+      <c r="H65" s="1" t="n"/>
+      <c r="I65" s="1" t="n"/>
+      <c r="J65" s="1" t="n"/>
+      <c r="K65" s="1" t="n"/>
+      <c r="L65" s="1" t="n"/>
+      <c r="M65" s="1" t="n"/>
+      <c r="N65" s="1" t="n"/>
+      <c r="O65" s="1" t="n"/>
       <c r="P65" s="7" t="inlineStr">
         <is>
           <t>טבלה</t>
@@ -47487,30 +47519,313 @@
         <v/>
       </c>
     </row>
+    <row r="910">
+      <c r="A910" s="4" t="n"/>
+      <c r="B910" s="4" t="n"/>
+      <c r="C910" s="4" t="n"/>
+      <c r="D910" s="4" t="n"/>
+      <c r="E910" s="4" t="n"/>
+      <c r="F910" s="4" t="n"/>
+      <c r="G910" s="4" t="n"/>
+      <c r="H910" s="4" t="n"/>
+      <c r="I910" s="4" t="n"/>
+      <c r="J910" s="4" t="n"/>
+      <c r="K910" s="4" t="n"/>
+      <c r="L910" s="4" t="n"/>
+      <c r="M910" s="4" t="n"/>
+      <c r="N910" s="4" t="n"/>
+      <c r="O910" s="4" t="n"/>
+      <c r="P910" s="7" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="Q910" s="8" t="inlineStr">
+        <is>
+          <t>T003O</t>
+        </is>
+      </c>
+      <c r="R910" s="7" t="inlineStr">
+        <is>
+          <t>T003O - סוגי פק"ע (Order Types; הוגדר כ-T350)</t>
+        </is>
+      </c>
+      <c r="S910" s="7" t="inlineStr"/>
+      <c r="T910" s="7" t="inlineStr">
+        <is>
+          <t>Config Guide</t>
+        </is>
+      </c>
+      <c r="U910" s="7" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="V910" s="9">
+        <f>HYPERLINK("#'"&amp;T910&amp;"'!"&amp;U910,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="4" t="n"/>
+      <c r="B911" s="4" t="n"/>
+      <c r="C911" s="4" t="n"/>
+      <c r="D911" s="4" t="n"/>
+      <c r="E911" s="4" t="n"/>
+      <c r="F911" s="4" t="n"/>
+      <c r="G911" s="4" t="n"/>
+      <c r="H911" s="4" t="n"/>
+      <c r="I911" s="4" t="n"/>
+      <c r="J911" s="4" t="n"/>
+      <c r="K911" s="4" t="n"/>
+      <c r="L911" s="4" t="n"/>
+      <c r="M911" s="4" t="n"/>
+      <c r="N911" s="4" t="n"/>
+      <c r="O911" s="4" t="n"/>
+      <c r="P911" s="7" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="Q911" s="8" t="inlineStr">
+        <is>
+          <t>T356</t>
+        </is>
+      </c>
+      <c r="R911" s="7" t="inlineStr">
+        <is>
+          <t>T356 - עדיפויות (Priorities)</t>
+        </is>
+      </c>
+      <c r="S911" s="7" t="inlineStr"/>
+      <c r="T911" s="7" t="inlineStr">
+        <is>
+          <t>Config Guide</t>
+        </is>
+      </c>
+      <c r="U911" s="7" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="V911" s="9">
+        <f>HYPERLINK("#'"&amp;T911&amp;"'!"&amp;U911,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="4" t="n"/>
+      <c r="B912" s="4" t="n"/>
+      <c r="C912" s="4" t="n"/>
+      <c r="D912" s="4" t="n"/>
+      <c r="E912" s="4" t="n"/>
+      <c r="F912" s="4" t="n"/>
+      <c r="G912" s="4" t="n"/>
+      <c r="H912" s="4" t="n"/>
+      <c r="I912" s="4" t="n"/>
+      <c r="J912" s="4" t="n"/>
+      <c r="K912" s="4" t="n"/>
+      <c r="L912" s="4" t="n"/>
+      <c r="M912" s="4" t="n"/>
+      <c r="N912" s="4" t="n"/>
+      <c r="O912" s="4" t="n"/>
+      <c r="P912" s="7" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="Q912" s="8" t="inlineStr">
+        <is>
+          <t>TQ80</t>
+        </is>
+      </c>
+      <c r="R912" s="7" t="inlineStr">
+        <is>
+          <t>TQ80 - סוגי הודעה (Notification Types)</t>
+        </is>
+      </c>
+      <c r="S912" s="7" t="inlineStr"/>
+      <c r="T912" s="7" t="inlineStr">
+        <is>
+          <t>Config Guide</t>
+        </is>
+      </c>
+      <c r="U912" s="7" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="V912" s="9">
+        <f>HYPERLINK("#'"&amp;T912&amp;"'!"&amp;U912,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="4" t="n"/>
+      <c r="B913" s="4" t="n"/>
+      <c r="C913" s="4" t="n"/>
+      <c r="D913" s="4" t="n"/>
+      <c r="E913" s="4" t="n"/>
+      <c r="F913" s="4" t="n"/>
+      <c r="G913" s="4" t="n"/>
+      <c r="H913" s="4" t="n"/>
+      <c r="I913" s="4" t="n"/>
+      <c r="J913" s="4" t="n"/>
+      <c r="K913" s="4" t="n"/>
+      <c r="L913" s="4" t="n"/>
+      <c r="M913" s="4" t="n"/>
+      <c r="N913" s="4" t="n"/>
+      <c r="O913" s="4" t="n"/>
+      <c r="P913" s="7" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="Q913" s="8" t="inlineStr">
+        <is>
+          <t>TJ30</t>
+        </is>
+      </c>
+      <c r="R913" s="7" t="inlineStr">
+        <is>
+          <t>TJ30 - פרופיל סטטוס משתמש (User Status Profile)</t>
+        </is>
+      </c>
+      <c r="S913" s="7" t="inlineStr"/>
+      <c r="T913" s="7" t="inlineStr">
+        <is>
+          <t>Config Guide</t>
+        </is>
+      </c>
+      <c r="U913" s="7" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="V913" s="9">
+        <f>HYPERLINK("#'"&amp;T913&amp;"'!"&amp;U913,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="4" t="n"/>
+      <c r="B914" s="4" t="n"/>
+      <c r="C914" s="4" t="n"/>
+      <c r="D914" s="4" t="n"/>
+      <c r="E914" s="4" t="n"/>
+      <c r="F914" s="4" t="n"/>
+      <c r="G914" s="4" t="n"/>
+      <c r="H914" s="4" t="n"/>
+      <c r="I914" s="4" t="n"/>
+      <c r="J914" s="4" t="n"/>
+      <c r="K914" s="4" t="n"/>
+      <c r="L914" s="4" t="n"/>
+      <c r="M914" s="4" t="n"/>
+      <c r="N914" s="4" t="n"/>
+      <c r="O914" s="4" t="n"/>
+      <c r="P914" s="7" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="Q914" s="8" t="inlineStr">
+        <is>
+          <t>TJ30T</t>
+        </is>
+      </c>
+      <c r="R914" s="7" t="inlineStr">
+        <is>
+          <t>TJ30T - טקסטים של סטטוס משתמש (User Status Texts)</t>
+        </is>
+      </c>
+      <c r="S914" s="7" t="inlineStr"/>
+      <c r="T914" s="7" t="inlineStr">
+        <is>
+          <t>Config Guide</t>
+        </is>
+      </c>
+      <c r="U914" s="7" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="V914" s="9">
+        <f>HYPERLINK("#'"&amp;T914&amp;"'!"&amp;U914,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="4" t="n"/>
+      <c r="B915" s="4" t="n"/>
+      <c r="C915" s="4" t="n"/>
+      <c r="D915" s="4" t="n"/>
+      <c r="E915" s="4" t="n"/>
+      <c r="F915" s="4" t="n"/>
+      <c r="G915" s="4" t="n"/>
+      <c r="H915" s="4" t="n"/>
+      <c r="I915" s="4" t="n"/>
+      <c r="J915" s="4" t="n"/>
+      <c r="K915" s="4" t="n"/>
+      <c r="L915" s="4" t="n"/>
+      <c r="M915" s="4" t="n"/>
+      <c r="N915" s="4" t="n"/>
+      <c r="O915" s="4" t="n"/>
+      <c r="P915" s="7" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="Q915" s="8" t="inlineStr">
+        <is>
+          <t>BUT000</t>
+        </is>
+      </c>
+      <c r="R915" s="7" t="inlineStr">
+        <is>
+          <t>BUT000 - שותף עסקי (Business Partner / Partner Profiles)</t>
+        </is>
+      </c>
+      <c r="S915" s="7" t="inlineStr"/>
+      <c r="T915" s="7" t="inlineStr">
+        <is>
+          <t>Config Guide</t>
+        </is>
+      </c>
+      <c r="U915" s="7" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="V915" s="9">
+        <f>HYPERLINK("#'"&amp;T915&amp;"'!"&amp;U915,"➜ פתח")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="26">
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="J2:O3"/>
     <mergeCell ref="F16:F17"/>
     <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="C28:F28"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="D13:D14"/>
     <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B25:H25"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="H19:H20"/>
     <mergeCell ref="F13:F14"/>
-    <mergeCell ref="B22:H22"/>
     <mergeCell ref="H13:H14"/>
     <mergeCell ref="H16:H17"/>
-    <mergeCell ref="B56:H60"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C25:F25"/>
     <mergeCell ref="D19:D20"/>
+    <mergeCell ref="B58:H62"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B22:B23"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="H10:H11"/>
@@ -47532,6 +47847,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId17"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.3" right="0.3" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
@@ -61969,6 +62285,341 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <printOptions horizontalCentered="1" gridLines="0"/>
+  <pageMargins left="0.3" right="0.3" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Segoe UI,Bold"&amp;13&amp;KD62027CBC ISRAEL&amp;C&amp;"Segoe UI,Bold"&amp;11&amp;K1E1E24Project NEO  |  SAP PM  ECC 6.0 -&gt; S/4HANA Migration&amp;R&amp;"Segoe UI"&amp;9&amp;K6B7280&amp;A</oddHeader>
+    <oddFooter>&amp;L&amp;"Segoe UI"&amp;8&amp;K6B7280SAP PM Migration Workbook  -  CBC Israel (Project NEO)&amp;C&amp;"Segoe UI"&amp;8&amp;K6B7280Page &amp;P of &amp;N&amp;R&amp;"Segoe UI"&amp;8&amp;K6B7280&amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001E1E24"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>◄ חזרה למסך הראשי</t>
+        </is>
+      </c>
+      <c r="B1" s="36" t="n"/>
+      <c r="C1" s="37" t="inlineStr">
+        <is>
+          <t>Config Guide  -  מדריך קונפיגורציה אנציקלופדי (SPRO)  ·  CBC NEO</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="73" t="inlineStr">
+        <is>
+          <t>מס' (#)</t>
+        </is>
+      </c>
+      <c r="B2" s="73" t="inlineStr">
+        <is>
+          <t>אובייקט קונפיגורציה (Object)</t>
+        </is>
+      </c>
+      <c r="C2" s="73" t="inlineStr">
+        <is>
+          <t>טרנזקציה (SPRO/T-code)</t>
+        </is>
+      </c>
+      <c r="D2" s="73" t="inlineStr">
+        <is>
+          <t>הסבר פונקציונלי בעברית (Configuration Guide)</t>
+        </is>
+      </c>
+      <c r="E2" s="73" t="inlineStr">
+        <is>
+          <t>תרגום מונחים (HE = EN)</t>
+        </is>
+      </c>
+      <c r="F2" s="73" t="inlineStr">
+        <is>
+          <t>SAP Help / Knowledge</t>
+        </is>
+      </c>
+      <c r="G2" s="73" t="inlineStr">
+        <is>
+          <t>Note / SIC / Fiori</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="118" customHeight="1">
+      <c r="A3" s="74" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="108" t="inlineStr">
+        <is>
+          <t>T003O - סוגי פק"ע (Order Types; הוגדר כ-T350)</t>
+        </is>
+      </c>
+      <c r="C3" s="109" t="inlineStr">
+        <is>
+          <t>SPRO; OIOA</t>
+        </is>
+      </c>
+      <c r="D3" s="75" t="inlineStr">
+        <is>
+          <t>מגדיר את סוגי פקודות העבודה (PM01 שגרתי, PM02 שירות חיצוני, PM03 השבתה). לכל סוג קובעים טווח מספרים, קטגוריית פקודה (30=PM), פרופיל סטטוס, פרופיל התחשבנות וברירות מחדל. נתיב SPRO: Plant Maintenance and Customer Service ◄ Maintenance and Service Orders ◄ Functions and Settings for Order Types ◄ Configure Order Types. ל-CBC: הפרדת סוגי פק"ע לפי זרם עבודה (מפעל/קו ייצור) מאפשרת בקרת עלות ודיווח נפרדים, והקצאת פרופיל סטטוס ייעודי לכל תהליך.</t>
+        </is>
+      </c>
+      <c r="E3" s="75" t="inlineStr">
+        <is>
+          <t>סוג פקודה = Order Type
+קטגוריית פקודה = Order Category
+טווח מספרים = Number Range
+פרופיל התחשבנות = Settlement Profile</t>
+        </is>
+      </c>
+      <c r="F3" s="110" t="inlineStr">
+        <is>
+          <t>SAP Help - PM Orders</t>
+        </is>
+      </c>
+      <c r="G3" s="110" t="inlineStr">
+        <is>
+          <t>SAP Community EAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="118" customHeight="1">
+      <c r="A4" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="111" t="inlineStr">
+        <is>
+          <t>T356 - עדיפויות (Priorities)</t>
+        </is>
+      </c>
+      <c r="C4" s="112" t="inlineStr">
+        <is>
+          <t>SPRO; OIOH</t>
+        </is>
+      </c>
+      <c r="D4" s="79" t="inlineStr">
+        <is>
+          <t>מגדיר את טבלת העדיפויות (1=דחוף ... 4=נמוך) וסוגי העדיפות (Priority Type) המקושרים לסוגי הודעה/פק"ע. לכל עדיפות נקבע מרווח זמן יחסי לחישוב אוטומטי של תאריך התחלה/סיום נדרש (Relative Start/End). ל-CBC: עדיפות 'תקלת קו ייצור' מתורגמת אוטומטית למועד טיפול מיידי (SLA), ומאפשרת ניטור הפרות SLA בדוחות PMIS.</t>
+        </is>
+      </c>
+      <c r="E4" s="79" t="inlineStr">
+        <is>
+          <t>עדיפות = Priority
+סוג עדיפות = Priority Type
+תאריך התחלה נדרש = Required Start
+מרווח יחסי = Relative Interval</t>
+        </is>
+      </c>
+      <c r="F4" s="113" t="inlineStr">
+        <is>
+          <t>SAP Help - Priorities</t>
+        </is>
+      </c>
+      <c r="G4" s="113" t="inlineStr">
+        <is>
+          <t>SAP Community EAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="118" customHeight="1">
+      <c r="A5" s="74" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="108" t="inlineStr">
+        <is>
+          <t>TQ80 - סוגי הודעה (Notification Types)</t>
+        </is>
+      </c>
+      <c r="C5" s="109" t="inlineStr">
+        <is>
+          <t>OIAL; SPRO, QCC0</t>
+        </is>
+      </c>
+      <c r="D5" s="75" t="inlineStr">
+        <is>
+          <t>מגדיר את סוגי הודעת האחזקה (M1 בקשה, M2 תקלה, M3 פעילות) ומקשר לכל סוג: פרופיל קטלוג (קודים מותרים), פריסת מסך (OIAL), סוג פק"ע ברירת מחדל וטווח מספרים. ל-CBC: הפרדה בין הודעת תקלה (M2) לבקשת שיפור (M1) מאפשרת ניתוח אמינות (MTBF/MTTR) נפרד וזרימת אישורים שונה לכל סוג.</t>
+        </is>
+      </c>
+      <c r="E5" s="75" t="inlineStr">
+        <is>
+          <t>סוג הודעה = Notification Type
+פרופיל קטלוג = Catalog Profile
+פריסת מסך = Screen Layout
+קבוצת קוד = Code Group</t>
+        </is>
+      </c>
+      <c r="F5" s="110" t="inlineStr">
+        <is>
+          <t>SAP Help - Notifications</t>
+        </is>
+      </c>
+      <c r="G5" s="110" t="inlineStr">
+        <is>
+          <t>Report Malfunction F2215</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="118" customHeight="1">
+      <c r="A6" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="111" t="inlineStr">
+        <is>
+          <t>TJ30 - פרופיל סטטוס משתמש (User Status Profile)</t>
+        </is>
+      </c>
+      <c r="C6" s="112" t="inlineStr">
+        <is>
+          <t>BS02; OIBS</t>
+        </is>
+      </c>
+      <c r="D6" s="79" t="inlineStr">
+        <is>
+          <t>מגדיר פרופיל סטטוס משתמש ובתוכו סטטוסים מותאמים אישית (למשל 'ממתין לחלקים', 'אושר תקציב') עם סדר מעבר, חסימה/התרה של תהליכים עסקיים (Business Transactions), וסטטוס ראשוני. נתיב: BS02. ל-CBC: סטטוס 'אישור בטיחות' חוסם שחרור פק"ע (REL) עד לאישור, ואוכף תהליך עבודה ארגוני מעבר לסטטוס המערכת הקבוע.</t>
+        </is>
+      </c>
+      <c r="E6" s="79" t="inlineStr">
+        <is>
+          <t>פרופיל סטטוס = Status Profile
+סטטוס משתמש = User Status
+תהליך עסקי = Business Transaction
+סטטוס ראשוני = Initial Status</t>
+        </is>
+      </c>
+      <c r="F6" s="113" t="inlineStr">
+        <is>
+          <t>SAP Help - Status Mgmt</t>
+        </is>
+      </c>
+      <c r="G6" s="113" t="inlineStr">
+        <is>
+          <t>SAP Community EAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="118" customHeight="1">
+      <c r="A7" s="74" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="108" t="inlineStr">
+        <is>
+          <t>TJ30T - טקסטים של סטטוס משתמש (User Status Texts)</t>
+        </is>
+      </c>
+      <c r="C7" s="109" t="inlineStr">
+        <is>
+          <t>BS02; BS03</t>
+        </is>
+      </c>
+      <c r="D7" s="75" t="inlineStr">
+        <is>
+          <t>מאחסן את הטקסטים הרב-לשוניים של סטטוסי המשתמש שהוגדרו ב-TJ30: קוד מקוצר (TXT04) ותיאור ארוך (TXT30) לפי שפה (SPRAS). ל-CBC: מאפשר תצוגת סטטוסים בעברית ובאנגלית לפי שפת המשתמש, וחיוני לדוחות דו-לשוניים ולממשקי Fiori.</t>
+        </is>
+      </c>
+      <c r="E7" s="75" t="inlineStr">
+        <is>
+          <t>טקסט סטטוס = Status Text
+קוד מקוצר = Short Code (TXT04)
+תיאור ארוך = Long Text (TXT30)
+שפה = Language Key</t>
+        </is>
+      </c>
+      <c r="F7" s="110" t="inlineStr">
+        <is>
+          <t>SAP Help - Status Texts</t>
+        </is>
+      </c>
+      <c r="G7" s="110" t="inlineStr">
+        <is>
+          <t>SAP Community EAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="118" customHeight="1">
+      <c r="A8" s="78" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="111" t="inlineStr">
+        <is>
+          <t>BUT000 - שותף עסקי (Business Partner / Partner Profiles)</t>
+        </is>
+      </c>
+      <c r="C8" s="112" t="inlineStr">
+        <is>
+          <t>BP; (ECC: XK01/MK01)</t>
+        </is>
+      </c>
+      <c r="D8" s="79" t="inlineStr">
+        <is>
+          <t>ב-S/4HANA ספקי שירותי האחזקה (קבלני משנה) מנוהלים כ-Business Partner (BP) במקום רשומת ספק קלאסית. נדרש CVI (Customer/Vendor Integration) להמרת LFA1 ל-BUT000 לפני/במהלך ההמרה. נתיב: tcode BP. ל-CBC: כל קבלן אחזקה חיצוני בפק"ע (פעולת PM02) חייב BP פעיל עם תפקיד ספק (FLVN00/FLVN01); היעדר CVI יכשיל את ה-Pre-Check של SUM. ראה SAP Note 2265093 (S4TWL - Business Partner Approach).</t>
+        </is>
+      </c>
+      <c r="E8" s="79" t="inlineStr">
+        <is>
+          <t>שותף עסקי = Business Partner
+תפקיד BP = BP Role
+קבוצת שותף = BP Grouping
+אינטגרציית ספק = CVI</t>
+        </is>
+      </c>
+      <c r="F8" s="113" t="inlineStr">
+        <is>
+          <t>SAP Note 2265093 (BP)</t>
+        </is>
+      </c>
+      <c r="G8" s="113" t="inlineStr">
+        <is>
+          <t>Simplification Item Catalog</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId13"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.3" right="0.3" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>

</xml_diff>